<commit_message>
adding gayatris figure code
</commit_message>
<xml_diff>
--- a/figures/landscape/curated_pathways.xlsx
+++ b/figures/landscape/curated_pathways.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10208"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ch57584/Documents/GitHub/precovid-analyses/figures/landscape/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ch57584/Documents/GitHub/MotrpacPreSuspensionAcute/figures/landscape/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50E0F6F2-31DA-7C49-AE13-5E428DCC8BCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A276099D-D53A-8D43-A496-69538922C979}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8120" yWindow="1920" windowWidth="28040" windowHeight="17180" activeTab="3" xr2:uid="{6CBD5D50-8479-BF41-8318-551E779FC86C}"/>
+    <workbookView xWindow="7420" yWindow="2160" windowWidth="28040" windowHeight="17180" activeTab="2" xr2:uid="{6CBD5D50-8479-BF41-8318-551E779FC86C}"/>
   </bookViews>
   <sheets>
     <sheet name="2B" sheetId="1" r:id="rId1"/>
     <sheet name="2F" sheetId="2" r:id="rId2"/>
-    <sheet name="3" sheetId="3" r:id="rId3"/>
-    <sheet name="5" sheetId="4" r:id="rId4"/>
+    <sheet name="S2E" sheetId="5" r:id="rId3"/>
+    <sheet name="3" sheetId="3" r:id="rId4"/>
+    <sheet name="5" sheetId="4" r:id="rId5"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="856" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1136" uniqueCount="145">
   <si>
     <t>GOBP_HEMOPOIESIS</t>
   </si>
@@ -363,6 +364,117 @@
   </si>
   <si>
     <t>AMPK (PRKAA1)</t>
+  </si>
+  <si>
+    <t>PTMSIGDB</t>
+  </si>
+  <si>
+    <t>PTMSIGDB_KINASE-iKiP</t>
+  </si>
+  <si>
+    <t>PTMSIGDB_KINASE-PSP</t>
+  </si>
+  <si>
+    <t>PTMSIGDB_KINASE-PSP_GSK3B</t>
+  </si>
+  <si>
+    <t>PTMSIGDB_KINASE-iKiP_MAPK12</t>
+  </si>
+  <si>
+    <t>PTMSIGDB_DISEASE-PSP</t>
+  </si>
+  <si>
+    <t>PTMSIGDB_DISEASE-PSP_Parkinsons_disease</t>
+  </si>
+  <si>
+    <t>PTMSIGDB_KINASE-PSP_mTOR/MTOR</t>
+  </si>
+  <si>
+    <t>PTMSIGDB_DISEASE-PSP_Alzheimers_disease</t>
+  </si>
+  <si>
+    <t>PTMSIGDB_PERT-PSP</t>
+  </si>
+  <si>
+    <t>PTMSIGDB_PERT-P100-DIA2</t>
+  </si>
+  <si>
+    <t>PTMSIGDB_PERT-P100-DIA2_ENDOTHELIN</t>
+  </si>
+  <si>
+    <t>PTMSIGDB_PATH-NP</t>
+  </si>
+  <si>
+    <t>PTMSIGDB_PATH-NP_TWEAK_PATHWAY</t>
+  </si>
+  <si>
+    <t>PTMSIGDB_PERT-P100-DIA2_BYL719</t>
+  </si>
+  <si>
+    <t>PTMSIGDB_PERT-PSP_TNF</t>
+  </si>
+  <si>
+    <t>Adipose_Muscle</t>
+  </si>
+  <si>
+    <t>PTMSIGDB_KINASE-iKiP_MAPK3.ERK1</t>
+  </si>
+  <si>
+    <t>PTMSIGDB_KINASE-iKiP_MAPK1.ERK2</t>
+  </si>
+  <si>
+    <t>PTMSIGDB_PERT-P100-DIA2_TRETINOIN</t>
+  </si>
+  <si>
+    <t>PTMSIGDB_PATH-BI</t>
+  </si>
+  <si>
+    <t>PTMSIGDB_PATH-BI_ISCHEMIA</t>
+  </si>
+  <si>
+    <t>PTMSIGDB_PERT-P100-DIA2_MOMELOTINIB</t>
+  </si>
+  <si>
+    <t>PTMSIGDB_DISEASE-PSP_PSP</t>
+  </si>
+  <si>
+    <t>PTMSIGDB_PERT-P100-DIA2_KN-93</t>
+  </si>
+  <si>
+    <t>PTMSIGDB_PERT-PSP_EGF</t>
+  </si>
+  <si>
+    <t>PTMSIGDB_DISEASE-PSP_DLB</t>
+  </si>
+  <si>
+    <t>PTMSIGDB_KINASE-iKiP_CDK5-CDK5R1p25</t>
+  </si>
+  <si>
+    <t>PTMSIGDB_PERT-PSP_SII_ANGIOTENSIN_2</t>
+  </si>
+  <si>
+    <t>PTMSIGDB_KINASE-iKiP_CDK1-CCNB1</t>
+  </si>
+  <si>
+    <t>PTMSIGDB_PERT-PSP_INSULIN</t>
+  </si>
+  <si>
+    <t>PTMSIGDB_PERT-PSP_RAPAMYCIN</t>
+  </si>
+  <si>
+    <t>PTMSIGDB_DISEASE-PSP_prostate_cancer</t>
+  </si>
+  <si>
+    <t>PTMSIGDB_PATH-NP_NOTCH_PATHWAY</t>
+  </si>
+  <si>
+    <t>PTMSIGDB_PATH-NP_TSLP_PATHWAY</t>
+  </si>
+  <si>
+    <t>PTMSIGDB_PERT-P100-DIA2_RO4929097</t>
+  </si>
+  <si>
+    <t>PTMSIGDB_KINASE-iKiP_MAP2K2</t>
   </si>
 </sst>
 </file>
@@ -8411,6 +8523,2557 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6973C21-7707-B645-8E5F-D6AB2ED24E75}">
+  <dimension ref="A1:O55"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I1" t="s">
+        <v>23</v>
+      </c>
+      <c r="J1" t="s">
+        <v>24</v>
+      </c>
+      <c r="K1" t="s">
+        <v>25</v>
+      </c>
+      <c r="L1" t="s">
+        <v>26</v>
+      </c>
+      <c r="M1" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" t="s">
+        <v>28</v>
+      </c>
+      <c r="O1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C2" t="s">
+        <v>109</v>
+      </c>
+      <c r="D2">
+        <v>15276</v>
+      </c>
+      <c r="E2" t="s">
+        <v>125</v>
+      </c>
+      <c r="F2" t="s">
+        <v>125</v>
+      </c>
+      <c r="G2">
+        <v>120</v>
+      </c>
+      <c r="H2">
+        <v>304</v>
+      </c>
+      <c r="I2">
+        <v>0.39500000000000002</v>
+      </c>
+      <c r="J2">
+        <v>66</v>
+      </c>
+      <c r="K2">
+        <v>3828</v>
+      </c>
+      <c r="L2">
+        <v>15657</v>
+      </c>
+      <c r="M2" s="1">
+        <v>6.3873599999999998E-13</v>
+      </c>
+      <c r="N2" s="1">
+        <v>3.05954E-10</v>
+      </c>
+      <c r="O2">
+        <v>12.1946786057447</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B3" t="s">
+        <v>108</v>
+      </c>
+      <c r="C3" t="s">
+        <v>109</v>
+      </c>
+      <c r="D3">
+        <v>15269</v>
+      </c>
+      <c r="E3" t="s">
+        <v>126</v>
+      </c>
+      <c r="F3" t="s">
+        <v>126</v>
+      </c>
+      <c r="G3">
+        <v>174</v>
+      </c>
+      <c r="H3">
+        <v>448</v>
+      </c>
+      <c r="I3">
+        <v>0.38800000000000001</v>
+      </c>
+      <c r="J3">
+        <v>79</v>
+      </c>
+      <c r="K3">
+        <v>3828</v>
+      </c>
+      <c r="L3">
+        <v>15657</v>
+      </c>
+      <c r="M3" s="1">
+        <v>1.13258E-9</v>
+      </c>
+      <c r="N3" s="1">
+        <v>1.08501E-7</v>
+      </c>
+      <c r="O3">
+        <v>8.9459311117597498</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B4" t="s">
+        <v>108</v>
+      </c>
+      <c r="C4" t="s">
+        <v>110</v>
+      </c>
+      <c r="D4">
+        <v>14946</v>
+      </c>
+      <c r="E4" t="s">
+        <v>111</v>
+      </c>
+      <c r="F4" t="s">
+        <v>111</v>
+      </c>
+      <c r="G4">
+        <v>54</v>
+      </c>
+      <c r="H4">
+        <v>362</v>
+      </c>
+      <c r="I4">
+        <v>0.14899999999999999</v>
+      </c>
+      <c r="J4">
+        <v>33</v>
+      </c>
+      <c r="K4">
+        <v>3828</v>
+      </c>
+      <c r="L4">
+        <v>15657</v>
+      </c>
+      <c r="M4" s="1">
+        <v>1.0918499999999999E-8</v>
+      </c>
+      <c r="N4" s="1">
+        <v>8.7165600000000001E-7</v>
+      </c>
+      <c r="O4">
+        <v>7.9618370215643202</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B5" t="s">
+        <v>108</v>
+      </c>
+      <c r="C5" t="s">
+        <v>109</v>
+      </c>
+      <c r="D5">
+        <v>15272</v>
+      </c>
+      <c r="E5" t="s">
+        <v>112</v>
+      </c>
+      <c r="F5" t="s">
+        <v>112</v>
+      </c>
+      <c r="G5">
+        <v>153</v>
+      </c>
+      <c r="H5">
+        <v>430</v>
+      </c>
+      <c r="I5">
+        <v>0.35599999999999998</v>
+      </c>
+      <c r="J5">
+        <v>69</v>
+      </c>
+      <c r="K5">
+        <v>3828</v>
+      </c>
+      <c r="L5">
+        <v>15657</v>
+      </c>
+      <c r="M5" s="1">
+        <v>1.7573600000000001E-8</v>
+      </c>
+      <c r="N5" s="1">
+        <v>1.20254E-6</v>
+      </c>
+      <c r="O5">
+        <v>7.7551392629791298</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" t="s">
+        <v>108</v>
+      </c>
+      <c r="C6" t="s">
+        <v>118</v>
+      </c>
+      <c r="D6">
+        <v>15580</v>
+      </c>
+      <c r="E6" t="s">
+        <v>127</v>
+      </c>
+      <c r="F6" t="s">
+        <v>127</v>
+      </c>
+      <c r="G6">
+        <v>107</v>
+      </c>
+      <c r="H6">
+        <v>225</v>
+      </c>
+      <c r="I6">
+        <v>0.47599999999999998</v>
+      </c>
+      <c r="J6">
+        <v>52</v>
+      </c>
+      <c r="K6">
+        <v>3828</v>
+      </c>
+      <c r="L6">
+        <v>15657</v>
+      </c>
+      <c r="M6" s="1">
+        <v>4.9566399999999997E-8</v>
+      </c>
+      <c r="N6" s="1">
+        <v>2.63803E-6</v>
+      </c>
+      <c r="O6">
+        <v>7.3048126226907799</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>40</v>
+      </c>
+      <c r="B7" t="s">
+        <v>108</v>
+      </c>
+      <c r="C7" t="s">
+        <v>128</v>
+      </c>
+      <c r="D7">
+        <v>15425</v>
+      </c>
+      <c r="E7" t="s">
+        <v>129</v>
+      </c>
+      <c r="F7" t="s">
+        <v>129</v>
+      </c>
+      <c r="G7">
+        <v>85</v>
+      </c>
+      <c r="H7">
+        <v>161</v>
+      </c>
+      <c r="I7">
+        <v>0.52800000000000002</v>
+      </c>
+      <c r="J7">
+        <v>43</v>
+      </c>
+      <c r="K7">
+        <v>3828</v>
+      </c>
+      <c r="L7">
+        <v>15657</v>
+      </c>
+      <c r="M7" s="1">
+        <v>1.6688900000000001E-7</v>
+      </c>
+      <c r="N7" s="1">
+        <v>7.2672599999999996E-6</v>
+      </c>
+      <c r="O7">
+        <v>6.77757228762714</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>40</v>
+      </c>
+      <c r="B8" t="s">
+        <v>108</v>
+      </c>
+      <c r="C8" t="s">
+        <v>118</v>
+      </c>
+      <c r="D8">
+        <v>15542</v>
+      </c>
+      <c r="E8" t="s">
+        <v>130</v>
+      </c>
+      <c r="F8" t="s">
+        <v>130</v>
+      </c>
+      <c r="G8">
+        <v>85</v>
+      </c>
+      <c r="H8">
+        <v>181</v>
+      </c>
+      <c r="I8">
+        <v>0.47</v>
+      </c>
+      <c r="J8">
+        <v>40</v>
+      </c>
+      <c r="K8">
+        <v>3828</v>
+      </c>
+      <c r="L8">
+        <v>15657</v>
+      </c>
+      <c r="M8" s="1">
+        <v>4.6692500000000002E-6</v>
+      </c>
+      <c r="N8">
+        <v>1.86381E-4</v>
+      </c>
+      <c r="O8">
+        <v>5.330752872543</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>40</v>
+      </c>
+      <c r="B9" t="s">
+        <v>108</v>
+      </c>
+      <c r="C9" t="s">
+        <v>113</v>
+      </c>
+      <c r="D9">
+        <v>14792</v>
+      </c>
+      <c r="E9" t="s">
+        <v>131</v>
+      </c>
+      <c r="F9" t="s">
+        <v>131</v>
+      </c>
+      <c r="G9">
+        <v>9</v>
+      </c>
+      <c r="H9">
+        <v>14</v>
+      </c>
+      <c r="I9">
+        <v>0.64300000000000002</v>
+      </c>
+      <c r="J9">
+        <v>8</v>
+      </c>
+      <c r="K9">
+        <v>3828</v>
+      </c>
+      <c r="L9">
+        <v>15657</v>
+      </c>
+      <c r="M9" s="1">
+        <v>8.9478600000000001E-5</v>
+      </c>
+      <c r="N9">
+        <v>2.381125E-3</v>
+      </c>
+      <c r="O9">
+        <v>4.0482808195802296</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>40</v>
+      </c>
+      <c r="B10" t="s">
+        <v>108</v>
+      </c>
+      <c r="C10" t="s">
+        <v>113</v>
+      </c>
+      <c r="D10">
+        <v>14793</v>
+      </c>
+      <c r="E10" t="s">
+        <v>114</v>
+      </c>
+      <c r="F10" t="s">
+        <v>114</v>
+      </c>
+      <c r="G10">
+        <v>18</v>
+      </c>
+      <c r="H10">
+        <v>47</v>
+      </c>
+      <c r="I10">
+        <v>0.38300000000000001</v>
+      </c>
+      <c r="J10">
+        <v>12</v>
+      </c>
+      <c r="K10">
+        <v>3828</v>
+      </c>
+      <c r="L10">
+        <v>15657</v>
+      </c>
+      <c r="M10">
+        <v>1.8230300000000001E-4</v>
+      </c>
+      <c r="N10">
+        <v>3.4929280000000002E-3</v>
+      </c>
+      <c r="O10">
+        <v>3.7392061844842099</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>40</v>
+      </c>
+      <c r="B11" t="s">
+        <v>108</v>
+      </c>
+      <c r="C11" t="s">
+        <v>110</v>
+      </c>
+      <c r="D11">
+        <v>15108</v>
+      </c>
+      <c r="E11" t="s">
+        <v>115</v>
+      </c>
+      <c r="F11" t="s">
+        <v>115</v>
+      </c>
+      <c r="G11">
+        <v>41</v>
+      </c>
+      <c r="H11">
+        <v>123</v>
+      </c>
+      <c r="I11">
+        <v>0.33300000000000002</v>
+      </c>
+      <c r="J11">
+        <v>21</v>
+      </c>
+      <c r="K11">
+        <v>3828</v>
+      </c>
+      <c r="L11">
+        <v>15657</v>
+      </c>
+      <c r="M11">
+        <v>1.9265499999999999E-4</v>
+      </c>
+      <c r="N11">
+        <v>3.5492969999999999E-3</v>
+      </c>
+      <c r="O11">
+        <v>3.71521971520415</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>40</v>
+      </c>
+      <c r="B12" t="s">
+        <v>108</v>
+      </c>
+      <c r="C12" t="s">
+        <v>118</v>
+      </c>
+      <c r="D12">
+        <v>15534</v>
+      </c>
+      <c r="E12" t="s">
+        <v>132</v>
+      </c>
+      <c r="F12" t="s">
+        <v>132</v>
+      </c>
+      <c r="G12">
+        <v>65</v>
+      </c>
+      <c r="H12">
+        <v>141</v>
+      </c>
+      <c r="I12">
+        <v>0.46100000000000002</v>
+      </c>
+      <c r="J12">
+        <v>29</v>
+      </c>
+      <c r="K12">
+        <v>3828</v>
+      </c>
+      <c r="L12">
+        <v>15657</v>
+      </c>
+      <c r="M12">
+        <v>2.9328200000000002E-4</v>
+      </c>
+      <c r="N12">
+        <v>4.6827409999999998E-3</v>
+      </c>
+      <c r="O12">
+        <v>3.5327145907547401</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>40</v>
+      </c>
+      <c r="B13" t="s">
+        <v>108</v>
+      </c>
+      <c r="C13" t="s">
+        <v>117</v>
+      </c>
+      <c r="D13">
+        <v>15644</v>
+      </c>
+      <c r="E13" t="s">
+        <v>133</v>
+      </c>
+      <c r="F13" t="s">
+        <v>133</v>
+      </c>
+      <c r="G13">
+        <v>53</v>
+      </c>
+      <c r="H13">
+        <v>162</v>
+      </c>
+      <c r="I13">
+        <v>0.32700000000000001</v>
+      </c>
+      <c r="J13">
+        <v>24</v>
+      </c>
+      <c r="K13">
+        <v>3828</v>
+      </c>
+      <c r="L13">
+        <v>15657</v>
+      </c>
+      <c r="M13">
+        <v>7.3243099999999997E-4</v>
+      </c>
+      <c r="N13">
+        <v>8.7378890000000004E-3</v>
+      </c>
+      <c r="O13">
+        <v>3.13523328255163</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>40</v>
+      </c>
+      <c r="B14" t="s">
+        <v>108</v>
+      </c>
+      <c r="C14" t="s">
+        <v>113</v>
+      </c>
+      <c r="D14">
+        <v>14776</v>
+      </c>
+      <c r="E14" t="s">
+        <v>116</v>
+      </c>
+      <c r="F14" t="s">
+        <v>116</v>
+      </c>
+      <c r="G14">
+        <v>39</v>
+      </c>
+      <c r="H14">
+        <v>130</v>
+      </c>
+      <c r="I14">
+        <v>0.3</v>
+      </c>
+      <c r="J14">
+        <v>19</v>
+      </c>
+      <c r="K14">
+        <v>3828</v>
+      </c>
+      <c r="L14">
+        <v>15657</v>
+      </c>
+      <c r="M14">
+        <v>8.61695E-4</v>
+      </c>
+      <c r="N14">
+        <v>9.4916600000000007E-3</v>
+      </c>
+      <c r="O14">
+        <v>3.0646464270482898</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>40</v>
+      </c>
+      <c r="B15" t="s">
+        <v>108</v>
+      </c>
+      <c r="C15" t="s">
+        <v>113</v>
+      </c>
+      <c r="D15">
+        <v>14780</v>
+      </c>
+      <c r="E15" t="s">
+        <v>134</v>
+      </c>
+      <c r="F15" t="s">
+        <v>134</v>
+      </c>
+      <c r="G15">
+        <v>9</v>
+      </c>
+      <c r="H15">
+        <v>15</v>
+      </c>
+      <c r="I15">
+        <v>0.6</v>
+      </c>
+      <c r="J15">
+        <v>7</v>
+      </c>
+      <c r="K15">
+        <v>3828</v>
+      </c>
+      <c r="L15">
+        <v>15657</v>
+      </c>
+      <c r="M15">
+        <v>1.159034E-3</v>
+      </c>
+      <c r="N15">
+        <v>1.1070323E-2</v>
+      </c>
+      <c r="O15">
+        <v>2.9359038239192299</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>40</v>
+      </c>
+      <c r="B16" t="s">
+        <v>108</v>
+      </c>
+      <c r="C16" t="s">
+        <v>118</v>
+      </c>
+      <c r="D16">
+        <v>15509</v>
+      </c>
+      <c r="E16" t="s">
+        <v>119</v>
+      </c>
+      <c r="F16" t="s">
+        <v>119</v>
+      </c>
+      <c r="G16">
+        <v>78</v>
+      </c>
+      <c r="H16">
+        <v>204</v>
+      </c>
+      <c r="I16">
+        <v>0.38200000000000001</v>
+      </c>
+      <c r="J16">
+        <v>31</v>
+      </c>
+      <c r="K16">
+        <v>3828</v>
+      </c>
+      <c r="L16">
+        <v>15657</v>
+      </c>
+      <c r="M16">
+        <v>1.9686040000000001E-3</v>
+      </c>
+      <c r="N16">
+        <v>1.6543177999999999E-2</v>
+      </c>
+      <c r="O16">
+        <v>2.7058416367878801</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>40</v>
+      </c>
+      <c r="B17" t="s">
+        <v>108</v>
+      </c>
+      <c r="C17" t="s">
+        <v>109</v>
+      </c>
+      <c r="D17">
+        <v>15153</v>
+      </c>
+      <c r="E17" t="s">
+        <v>135</v>
+      </c>
+      <c r="F17" t="s">
+        <v>135</v>
+      </c>
+      <c r="G17">
+        <v>73</v>
+      </c>
+      <c r="H17">
+        <v>190</v>
+      </c>
+      <c r="I17">
+        <v>0.38400000000000001</v>
+      </c>
+      <c r="J17">
+        <v>29</v>
+      </c>
+      <c r="K17">
+        <v>3828</v>
+      </c>
+      <c r="L17">
+        <v>15657</v>
+      </c>
+      <c r="M17">
+        <v>2.7279800000000001E-3</v>
+      </c>
+      <c r="N17">
+        <v>2.0417223000000002E-2</v>
+      </c>
+      <c r="O17">
+        <v>2.56415881800437</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>40</v>
+      </c>
+      <c r="B18" t="s">
+        <v>108</v>
+      </c>
+      <c r="C18" t="s">
+        <v>117</v>
+      </c>
+      <c r="D18">
+        <v>15708</v>
+      </c>
+      <c r="E18" t="s">
+        <v>136</v>
+      </c>
+      <c r="F18" t="s">
+        <v>136</v>
+      </c>
+      <c r="G18">
+        <v>28</v>
+      </c>
+      <c r="H18">
+        <v>33</v>
+      </c>
+      <c r="I18">
+        <v>0.84799999999999998</v>
+      </c>
+      <c r="J18">
+        <v>14</v>
+      </c>
+      <c r="K18">
+        <v>3828</v>
+      </c>
+      <c r="L18">
+        <v>15657</v>
+      </c>
+      <c r="M18">
+        <v>3.0065700000000001E-3</v>
+      </c>
+      <c r="N18">
+        <v>2.2101272000000002E-2</v>
+      </c>
+      <c r="O18">
+        <v>2.5219286803068099</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>40</v>
+      </c>
+      <c r="B19" t="s">
+        <v>108</v>
+      </c>
+      <c r="C19" t="s">
+        <v>120</v>
+      </c>
+      <c r="D19">
+        <v>15458</v>
+      </c>
+      <c r="E19" t="s">
+        <v>121</v>
+      </c>
+      <c r="F19" t="s">
+        <v>121</v>
+      </c>
+      <c r="G19">
+        <v>10</v>
+      </c>
+      <c r="H19">
+        <v>18</v>
+      </c>
+      <c r="I19">
+        <v>0.55600000000000005</v>
+      </c>
+      <c r="J19">
+        <v>7</v>
+      </c>
+      <c r="K19">
+        <v>3828</v>
+      </c>
+      <c r="L19">
+        <v>15657</v>
+      </c>
+      <c r="M19">
+        <v>3.0452690000000002E-3</v>
+      </c>
+      <c r="N19">
+        <v>2.2101272000000002E-2</v>
+      </c>
+      <c r="O19">
+        <v>2.5163743384808002</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>40</v>
+      </c>
+      <c r="B20" t="s">
+        <v>108</v>
+      </c>
+      <c r="C20" t="s">
+        <v>109</v>
+      </c>
+      <c r="D20">
+        <v>15146</v>
+      </c>
+      <c r="E20" t="s">
+        <v>137</v>
+      </c>
+      <c r="F20" t="s">
+        <v>137</v>
+      </c>
+      <c r="G20">
+        <v>93</v>
+      </c>
+      <c r="H20">
+        <v>253</v>
+      </c>
+      <c r="I20">
+        <v>0.36799999999999999</v>
+      </c>
+      <c r="J20">
+        <v>35</v>
+      </c>
+      <c r="K20">
+        <v>3828</v>
+      </c>
+      <c r="L20">
+        <v>15657</v>
+      </c>
+      <c r="M20">
+        <v>3.1279989999999998E-3</v>
+      </c>
+      <c r="N20">
+        <v>2.2362861000000001E-2</v>
+      </c>
+      <c r="O20">
+        <v>2.5047333944531598</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>40</v>
+      </c>
+      <c r="B21" t="s">
+        <v>108</v>
+      </c>
+      <c r="C21" t="s">
+        <v>117</v>
+      </c>
+      <c r="D21">
+        <v>15678</v>
+      </c>
+      <c r="E21" t="s">
+        <v>138</v>
+      </c>
+      <c r="F21" t="s">
+        <v>138</v>
+      </c>
+      <c r="G21">
+        <v>37</v>
+      </c>
+      <c r="H21">
+        <v>75</v>
+      </c>
+      <c r="I21">
+        <v>0.49299999999999999</v>
+      </c>
+      <c r="J21">
+        <v>17</v>
+      </c>
+      <c r="K21">
+        <v>3828</v>
+      </c>
+      <c r="L21">
+        <v>15657</v>
+      </c>
+      <c r="M21">
+        <v>3.503146E-3</v>
+      </c>
+      <c r="N21">
+        <v>2.4620548999999999E-2</v>
+      </c>
+      <c r="O21">
+        <v>2.4555417622903501</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>40</v>
+      </c>
+      <c r="B22" t="s">
+        <v>108</v>
+      </c>
+      <c r="C22" t="s">
+        <v>117</v>
+      </c>
+      <c r="D22">
+        <v>15703</v>
+      </c>
+      <c r="E22" t="s">
+        <v>139</v>
+      </c>
+      <c r="F22" t="s">
+        <v>139</v>
+      </c>
+      <c r="G22">
+        <v>15</v>
+      </c>
+      <c r="H22">
+        <v>36</v>
+      </c>
+      <c r="I22">
+        <v>0.41699999999999998</v>
+      </c>
+      <c r="J22">
+        <v>9</v>
+      </c>
+      <c r="K22">
+        <v>3828</v>
+      </c>
+      <c r="L22">
+        <v>15657</v>
+      </c>
+      <c r="M22">
+        <v>3.5465929999999998E-3</v>
+      </c>
+      <c r="N22">
+        <v>2.4620548999999999E-2</v>
+      </c>
+      <c r="O22">
+        <v>2.4501886474445902</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>40</v>
+      </c>
+      <c r="B23" t="s">
+        <v>108</v>
+      </c>
+      <c r="C23" t="s">
+        <v>118</v>
+      </c>
+      <c r="D23">
+        <v>15487</v>
+      </c>
+      <c r="E23" t="s">
+        <v>122</v>
+      </c>
+      <c r="F23" t="s">
+        <v>122</v>
+      </c>
+      <c r="G23">
+        <v>59</v>
+      </c>
+      <c r="H23">
+        <v>141</v>
+      </c>
+      <c r="I23">
+        <v>0.41799999999999998</v>
+      </c>
+      <c r="J23">
+        <v>24</v>
+      </c>
+      <c r="K23">
+        <v>3828</v>
+      </c>
+      <c r="L23">
+        <v>15657</v>
+      </c>
+      <c r="M23">
+        <v>4.2771620000000002E-3</v>
+      </c>
+      <c r="N23">
+        <v>2.8663912999999999E-2</v>
+      </c>
+      <c r="O23">
+        <v>2.36884430027541</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>40</v>
+      </c>
+      <c r="B24" t="s">
+        <v>108</v>
+      </c>
+      <c r="C24" t="s">
+        <v>113</v>
+      </c>
+      <c r="D24">
+        <v>14844</v>
+      </c>
+      <c r="E24" t="s">
+        <v>140</v>
+      </c>
+      <c r="F24" t="s">
+        <v>140</v>
+      </c>
+      <c r="G24">
+        <v>13</v>
+      </c>
+      <c r="H24">
+        <v>58</v>
+      </c>
+      <c r="I24">
+        <v>0.224</v>
+      </c>
+      <c r="J24">
+        <v>8</v>
+      </c>
+      <c r="K24">
+        <v>3828</v>
+      </c>
+      <c r="L24">
+        <v>15657</v>
+      </c>
+      <c r="M24">
+        <v>4.8575579999999997E-3</v>
+      </c>
+      <c r="N24">
+        <v>3.1442843999999998E-2</v>
+      </c>
+      <c r="O24">
+        <v>2.3135820051533802</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>40</v>
+      </c>
+      <c r="B25" t="s">
+        <v>108</v>
+      </c>
+      <c r="C25" t="s">
+        <v>120</v>
+      </c>
+      <c r="D25">
+        <v>15449</v>
+      </c>
+      <c r="E25" t="s">
+        <v>141</v>
+      </c>
+      <c r="F25" t="s">
+        <v>141</v>
+      </c>
+      <c r="G25">
+        <v>11</v>
+      </c>
+      <c r="H25">
+        <v>30</v>
+      </c>
+      <c r="I25">
+        <v>0.36699999999999999</v>
+      </c>
+      <c r="J25">
+        <v>7</v>
+      </c>
+      <c r="K25">
+        <v>3828</v>
+      </c>
+      <c r="L25">
+        <v>15657</v>
+      </c>
+      <c r="M25">
+        <v>6.6093100000000002E-3</v>
+      </c>
+      <c r="N25">
+        <v>3.8608041000000003E-2</v>
+      </c>
+      <c r="O25">
+        <v>2.1798438777056002</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>40</v>
+      </c>
+      <c r="B26" t="s">
+        <v>108</v>
+      </c>
+      <c r="C26" t="s">
+        <v>117</v>
+      </c>
+      <c r="D26">
+        <v>15719</v>
+      </c>
+      <c r="E26" t="s">
+        <v>123</v>
+      </c>
+      <c r="F26" t="s">
+        <v>123</v>
+      </c>
+      <c r="G26">
+        <v>11</v>
+      </c>
+      <c r="H26">
+        <v>31</v>
+      </c>
+      <c r="I26">
+        <v>0.35499999999999998</v>
+      </c>
+      <c r="J26">
+        <v>7</v>
+      </c>
+      <c r="K26">
+        <v>3828</v>
+      </c>
+      <c r="L26">
+        <v>15657</v>
+      </c>
+      <c r="M26">
+        <v>6.6093100000000002E-3</v>
+      </c>
+      <c r="N26">
+        <v>3.8608041000000003E-2</v>
+      </c>
+      <c r="O26">
+        <v>2.1798438777056002</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>40</v>
+      </c>
+      <c r="B27" t="s">
+        <v>108</v>
+      </c>
+      <c r="C27" t="s">
+        <v>120</v>
+      </c>
+      <c r="D27">
+        <v>15457</v>
+      </c>
+      <c r="E27" t="s">
+        <v>142</v>
+      </c>
+      <c r="F27" t="s">
+        <v>142</v>
+      </c>
+      <c r="G27">
+        <v>55</v>
+      </c>
+      <c r="H27">
+        <v>173</v>
+      </c>
+      <c r="I27">
+        <v>0.318</v>
+      </c>
+      <c r="J27">
+        <v>22</v>
+      </c>
+      <c r="K27">
+        <v>3828</v>
+      </c>
+      <c r="L27">
+        <v>15657</v>
+      </c>
+      <c r="M27">
+        <v>7.6805019999999996E-3</v>
+      </c>
+      <c r="N27">
+        <v>4.3462537000000002E-2</v>
+      </c>
+      <c r="O27">
+        <v>2.11461039341836</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>40</v>
+      </c>
+      <c r="B28" t="s">
+        <v>108</v>
+      </c>
+      <c r="C28" t="s">
+        <v>118</v>
+      </c>
+      <c r="D28">
+        <v>15560</v>
+      </c>
+      <c r="E28" t="s">
+        <v>143</v>
+      </c>
+      <c r="F28" t="s">
+        <v>143</v>
+      </c>
+      <c r="G28">
+        <v>86</v>
+      </c>
+      <c r="H28">
+        <v>198</v>
+      </c>
+      <c r="I28">
+        <v>0.434</v>
+      </c>
+      <c r="J28">
+        <v>24</v>
+      </c>
+      <c r="K28">
+        <v>3828</v>
+      </c>
+      <c r="L28">
+        <v>15657</v>
+      </c>
+      <c r="M28">
+        <v>0.262678525</v>
+      </c>
+      <c r="N28">
+        <v>0.50329205499999996</v>
+      </c>
+      <c r="O28">
+        <v>0.58057543104044795</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>40</v>
+      </c>
+      <c r="B29" t="s">
+        <v>108</v>
+      </c>
+      <c r="C29" t="s">
+        <v>109</v>
+      </c>
+      <c r="D29">
+        <v>15251</v>
+      </c>
+      <c r="E29" t="s">
+        <v>144</v>
+      </c>
+      <c r="F29" t="s">
+        <v>144</v>
+      </c>
+      <c r="G29">
+        <v>13</v>
+      </c>
+      <c r="H29">
+        <v>24</v>
+      </c>
+      <c r="I29">
+        <v>0.54200000000000004</v>
+      </c>
+      <c r="J29">
+        <v>2</v>
+      </c>
+      <c r="K29">
+        <v>3828</v>
+      </c>
+      <c r="L29">
+        <v>15657</v>
+      </c>
+      <c r="M29">
+        <v>0.86405846900000005</v>
+      </c>
+      <c r="N29">
+        <v>0.94064546999999998</v>
+      </c>
+      <c r="O29">
+        <v>6.3456868742280501E-2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>77</v>
+      </c>
+      <c r="B30" t="s">
+        <v>108</v>
+      </c>
+      <c r="C30" t="s">
+        <v>109</v>
+      </c>
+      <c r="D30">
+        <v>15251</v>
+      </c>
+      <c r="E30" t="s">
+        <v>144</v>
+      </c>
+      <c r="F30" t="s">
+        <v>144</v>
+      </c>
+      <c r="G30">
+        <v>12</v>
+      </c>
+      <c r="H30">
+        <v>24</v>
+      </c>
+      <c r="I30">
+        <v>0.5</v>
+      </c>
+      <c r="J30">
+        <v>3</v>
+      </c>
+      <c r="K30">
+        <v>229</v>
+      </c>
+      <c r="L30">
+        <v>7217</v>
+      </c>
+      <c r="M30">
+        <v>5.6100380000000004E-3</v>
+      </c>
+      <c r="N30">
+        <v>0.82959132300000005</v>
+      </c>
+      <c r="O30">
+        <v>2.25103419700865</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>77</v>
+      </c>
+      <c r="B31" t="s">
+        <v>108</v>
+      </c>
+      <c r="C31" t="s">
+        <v>109</v>
+      </c>
+      <c r="D31">
+        <v>15153</v>
+      </c>
+      <c r="E31" t="s">
+        <v>135</v>
+      </c>
+      <c r="F31" t="s">
+        <v>135</v>
+      </c>
+      <c r="G31">
+        <v>50</v>
+      </c>
+      <c r="H31">
+        <v>190</v>
+      </c>
+      <c r="I31">
+        <v>0.26300000000000001</v>
+      </c>
+      <c r="J31">
+        <v>3</v>
+      </c>
+      <c r="K31">
+        <v>229</v>
+      </c>
+      <c r="L31">
+        <v>7217</v>
+      </c>
+      <c r="M31">
+        <v>0.21100380899999999</v>
+      </c>
+      <c r="N31">
+        <v>0.88569962599999996</v>
+      </c>
+      <c r="O31">
+        <v>0.67570970483145198</v>
+      </c>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>77</v>
+      </c>
+      <c r="B32" t="s">
+        <v>108</v>
+      </c>
+      <c r="C32" t="s">
+        <v>128</v>
+      </c>
+      <c r="D32">
+        <v>15425</v>
+      </c>
+      <c r="E32" t="s">
+        <v>129</v>
+      </c>
+      <c r="F32" t="s">
+        <v>129</v>
+      </c>
+      <c r="G32">
+        <v>64</v>
+      </c>
+      <c r="H32">
+        <v>161</v>
+      </c>
+      <c r="I32">
+        <v>0.39800000000000002</v>
+      </c>
+      <c r="J32">
+        <v>3</v>
+      </c>
+      <c r="K32">
+        <v>229</v>
+      </c>
+      <c r="L32">
+        <v>7217</v>
+      </c>
+      <c r="M32">
+        <v>0.33175828200000002</v>
+      </c>
+      <c r="N32">
+        <v>0.88569962599999996</v>
+      </c>
+      <c r="O32">
+        <v>0.47917822661875398</v>
+      </c>
+    </row>
+    <row r="33" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>77</v>
+      </c>
+      <c r="B33" t="s">
+        <v>108</v>
+      </c>
+      <c r="C33" t="s">
+        <v>118</v>
+      </c>
+      <c r="D33">
+        <v>15560</v>
+      </c>
+      <c r="E33" t="s">
+        <v>143</v>
+      </c>
+      <c r="F33" t="s">
+        <v>143</v>
+      </c>
+      <c r="G33">
+        <v>68</v>
+      </c>
+      <c r="H33">
+        <v>198</v>
+      </c>
+      <c r="I33">
+        <v>0.34300000000000003</v>
+      </c>
+      <c r="J33">
+        <v>3</v>
+      </c>
+      <c r="K33">
+        <v>229</v>
+      </c>
+      <c r="L33">
+        <v>7217</v>
+      </c>
+      <c r="M33">
+        <v>0.36674844200000001</v>
+      </c>
+      <c r="N33">
+        <v>0.88569962599999996</v>
+      </c>
+      <c r="O33">
+        <v>0.43563172242602899</v>
+      </c>
+    </row>
+    <row r="34" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>77</v>
+      </c>
+      <c r="B34" t="s">
+        <v>108</v>
+      </c>
+      <c r="C34" t="s">
+        <v>120</v>
+      </c>
+      <c r="D34">
+        <v>15457</v>
+      </c>
+      <c r="E34" t="s">
+        <v>142</v>
+      </c>
+      <c r="F34" t="s">
+        <v>142</v>
+      </c>
+      <c r="G34">
+        <v>49</v>
+      </c>
+      <c r="H34">
+        <v>173</v>
+      </c>
+      <c r="I34">
+        <v>0.28299999999999997</v>
+      </c>
+      <c r="J34">
+        <v>2</v>
+      </c>
+      <c r="K34">
+        <v>229</v>
+      </c>
+      <c r="L34">
+        <v>7217</v>
+      </c>
+      <c r="M34">
+        <v>0.46387761199999999</v>
+      </c>
+      <c r="N34">
+        <v>0.88569962599999996</v>
+      </c>
+      <c r="O34">
+        <v>0.33359658721283297</v>
+      </c>
+    </row>
+    <row r="35" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>77</v>
+      </c>
+      <c r="B35" t="s">
+        <v>108</v>
+      </c>
+      <c r="C35" t="s">
+        <v>118</v>
+      </c>
+      <c r="D35">
+        <v>15534</v>
+      </c>
+      <c r="E35" t="s">
+        <v>132</v>
+      </c>
+      <c r="F35" t="s">
+        <v>132</v>
+      </c>
+      <c r="G35">
+        <v>50</v>
+      </c>
+      <c r="H35">
+        <v>141</v>
+      </c>
+      <c r="I35">
+        <v>0.35499999999999998</v>
+      </c>
+      <c r="J35">
+        <v>2</v>
+      </c>
+      <c r="K35">
+        <v>229</v>
+      </c>
+      <c r="L35">
+        <v>7217</v>
+      </c>
+      <c r="M35">
+        <v>0.47441401999999999</v>
+      </c>
+      <c r="N35">
+        <v>0.88569962599999996</v>
+      </c>
+      <c r="O35">
+        <v>0.323842485076622</v>
+      </c>
+    </row>
+    <row r="36" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>77</v>
+      </c>
+      <c r="B36" t="s">
+        <v>108</v>
+      </c>
+      <c r="C36" t="s">
+        <v>118</v>
+      </c>
+      <c r="D36">
+        <v>15487</v>
+      </c>
+      <c r="E36" t="s">
+        <v>122</v>
+      </c>
+      <c r="F36" t="s">
+        <v>122</v>
+      </c>
+      <c r="G36">
+        <v>51</v>
+      </c>
+      <c r="H36">
+        <v>141</v>
+      </c>
+      <c r="I36">
+        <v>0.36199999999999999</v>
+      </c>
+      <c r="J36">
+        <v>2</v>
+      </c>
+      <c r="K36">
+        <v>229</v>
+      </c>
+      <c r="L36">
+        <v>7217</v>
+      </c>
+      <c r="M36">
+        <v>0.48482492799999999</v>
+      </c>
+      <c r="N36">
+        <v>0.88569962599999996</v>
+      </c>
+      <c r="O36">
+        <v>0.31441505836627498</v>
+      </c>
+    </row>
+    <row r="37" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>77</v>
+      </c>
+      <c r="B37" t="s">
+        <v>108</v>
+      </c>
+      <c r="C37" t="s">
+        <v>117</v>
+      </c>
+      <c r="D37">
+        <v>15708</v>
+      </c>
+      <c r="E37" t="s">
+        <v>136</v>
+      </c>
+      <c r="F37" t="s">
+        <v>136</v>
+      </c>
+      <c r="G37">
+        <v>22</v>
+      </c>
+      <c r="H37">
+        <v>33</v>
+      </c>
+      <c r="I37">
+        <v>0.66700000000000004</v>
+      </c>
+      <c r="J37">
+        <v>1</v>
+      </c>
+      <c r="K37">
+        <v>229</v>
+      </c>
+      <c r="L37">
+        <v>7217</v>
+      </c>
+      <c r="M37">
+        <v>0.50857217200000004</v>
+      </c>
+      <c r="N37">
+        <v>0.88569962599999996</v>
+      </c>
+      <c r="O37">
+        <v>0.29364740719114801</v>
+      </c>
+    </row>
+    <row r="38" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>77</v>
+      </c>
+      <c r="B38" t="s">
+        <v>108</v>
+      </c>
+      <c r="C38" t="s">
+        <v>109</v>
+      </c>
+      <c r="D38">
+        <v>15276</v>
+      </c>
+      <c r="E38" t="s">
+        <v>125</v>
+      </c>
+      <c r="F38" t="s">
+        <v>125</v>
+      </c>
+      <c r="G38">
+        <v>90</v>
+      </c>
+      <c r="H38">
+        <v>304</v>
+      </c>
+      <c r="I38">
+        <v>0.29599999999999999</v>
+      </c>
+      <c r="J38">
+        <v>3</v>
+      </c>
+      <c r="K38">
+        <v>229</v>
+      </c>
+      <c r="L38">
+        <v>7217</v>
+      </c>
+      <c r="M38">
+        <v>0.548202203</v>
+      </c>
+      <c r="N38">
+        <v>0.88569962599999996</v>
+      </c>
+      <c r="O38">
+        <v>0.26105922354146499</v>
+      </c>
+    </row>
+    <row r="39" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>77</v>
+      </c>
+      <c r="B39" t="s">
+        <v>108</v>
+      </c>
+      <c r="C39" t="s">
+        <v>118</v>
+      </c>
+      <c r="D39">
+        <v>15509</v>
+      </c>
+      <c r="E39" t="s">
+        <v>119</v>
+      </c>
+      <c r="F39" t="s">
+        <v>119</v>
+      </c>
+      <c r="G39">
+        <v>59</v>
+      </c>
+      <c r="H39">
+        <v>204</v>
+      </c>
+      <c r="I39">
+        <v>0.28899999999999998</v>
+      </c>
+      <c r="J39">
+        <v>2</v>
+      </c>
+      <c r="K39">
+        <v>229</v>
+      </c>
+      <c r="L39">
+        <v>7217</v>
+      </c>
+      <c r="M39">
+        <v>0.56333195800000002</v>
+      </c>
+      <c r="N39">
+        <v>0.88569962599999996</v>
+      </c>
+      <c r="O39">
+        <v>0.249235610402569</v>
+      </c>
+    </row>
+    <row r="40" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>77</v>
+      </c>
+      <c r="B40" t="s">
+        <v>108</v>
+      </c>
+      <c r="C40" t="s">
+        <v>109</v>
+      </c>
+      <c r="D40">
+        <v>15269</v>
+      </c>
+      <c r="E40" t="s">
+        <v>126</v>
+      </c>
+      <c r="F40" t="s">
+        <v>126</v>
+      </c>
+      <c r="G40">
+        <v>127</v>
+      </c>
+      <c r="H40">
+        <v>448</v>
+      </c>
+      <c r="I40">
+        <v>0.28299999999999997</v>
+      </c>
+      <c r="J40">
+        <v>4</v>
+      </c>
+      <c r="K40">
+        <v>229</v>
+      </c>
+      <c r="L40">
+        <v>7217</v>
+      </c>
+      <c r="M40">
+        <v>0.57729903599999999</v>
+      </c>
+      <c r="N40">
+        <v>0.88569962599999996</v>
+      </c>
+      <c r="O40">
+        <v>0.23859916770530101</v>
+      </c>
+    </row>
+    <row r="41" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>77</v>
+      </c>
+      <c r="B41" t="s">
+        <v>108</v>
+      </c>
+      <c r="C41" t="s">
+        <v>109</v>
+      </c>
+      <c r="D41">
+        <v>15146</v>
+      </c>
+      <c r="E41" t="s">
+        <v>137</v>
+      </c>
+      <c r="F41" t="s">
+        <v>137</v>
+      </c>
+      <c r="G41">
+        <v>66</v>
+      </c>
+      <c r="H41">
+        <v>253</v>
+      </c>
+      <c r="I41">
+        <v>0.26100000000000001</v>
+      </c>
+      <c r="J41">
+        <v>2</v>
+      </c>
+      <c r="K41">
+        <v>229</v>
+      </c>
+      <c r="L41">
+        <v>7217</v>
+      </c>
+      <c r="M41">
+        <v>0.62472418200000002</v>
+      </c>
+      <c r="N41">
+        <v>0.88569962599999996</v>
+      </c>
+      <c r="O41">
+        <v>0.20431168293520199</v>
+      </c>
+    </row>
+    <row r="42" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>77</v>
+      </c>
+      <c r="B42" t="s">
+        <v>108</v>
+      </c>
+      <c r="C42" t="s">
+        <v>118</v>
+      </c>
+      <c r="D42">
+        <v>15542</v>
+      </c>
+      <c r="E42" t="s">
+        <v>130</v>
+      </c>
+      <c r="F42" t="s">
+        <v>130</v>
+      </c>
+      <c r="G42">
+        <v>69</v>
+      </c>
+      <c r="H42">
+        <v>181</v>
+      </c>
+      <c r="I42">
+        <v>0.38100000000000001</v>
+      </c>
+      <c r="J42">
+        <v>1</v>
+      </c>
+      <c r="K42">
+        <v>229</v>
+      </c>
+      <c r="L42">
+        <v>7217</v>
+      </c>
+      <c r="M42">
+        <v>0.89307460500000002</v>
+      </c>
+      <c r="N42">
+        <v>0.91120809999999997</v>
+      </c>
+      <c r="O42">
+        <v>4.91122598276253E-2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>77</v>
+      </c>
+      <c r="B43" t="s">
+        <v>108</v>
+      </c>
+      <c r="C43" t="s">
+        <v>118</v>
+      </c>
+      <c r="D43">
+        <v>15580</v>
+      </c>
+      <c r="E43" t="s">
+        <v>127</v>
+      </c>
+      <c r="F43" t="s">
+        <v>127</v>
+      </c>
+      <c r="G43">
+        <v>83</v>
+      </c>
+      <c r="H43">
+        <v>225</v>
+      </c>
+      <c r="I43">
+        <v>0.36899999999999999</v>
+      </c>
+      <c r="J43">
+        <v>1</v>
+      </c>
+      <c r="K43">
+        <v>229</v>
+      </c>
+      <c r="L43">
+        <v>7217</v>
+      </c>
+      <c r="M43">
+        <v>0.93224822900000004</v>
+      </c>
+      <c r="N43">
+        <v>0.94161755800000002</v>
+      </c>
+      <c r="O43">
+        <v>3.0468432998844001E-2</v>
+      </c>
+    </row>
+    <row r="44" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>124</v>
+      </c>
+      <c r="B44" t="s">
+        <v>108</v>
+      </c>
+      <c r="C44" t="s">
+        <v>118</v>
+      </c>
+      <c r="D44">
+        <v>15487</v>
+      </c>
+      <c r="E44" t="s">
+        <v>122</v>
+      </c>
+      <c r="F44" t="s">
+        <v>122</v>
+      </c>
+      <c r="G44">
+        <v>59</v>
+      </c>
+      <c r="H44">
+        <v>141</v>
+      </c>
+      <c r="I44">
+        <v>0.41799999999999998</v>
+      </c>
+      <c r="J44">
+        <v>4</v>
+      </c>
+      <c r="K44">
+        <v>36</v>
+      </c>
+      <c r="L44">
+        <v>15657</v>
+      </c>
+      <c r="M44" s="1">
+        <v>9.7891900000000004E-6</v>
+      </c>
+      <c r="N44">
+        <v>1.4585889999999999E-3</v>
+      </c>
+      <c r="O44">
+        <v>5.0092532421175804</v>
+      </c>
+    </row>
+    <row r="45" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>124</v>
+      </c>
+      <c r="B45" t="s">
+        <v>108</v>
+      </c>
+      <c r="C45" t="s">
+        <v>118</v>
+      </c>
+      <c r="D45">
+        <v>15560</v>
+      </c>
+      <c r="E45" t="s">
+        <v>143</v>
+      </c>
+      <c r="F45" t="s">
+        <v>143</v>
+      </c>
+      <c r="G45">
+        <v>86</v>
+      </c>
+      <c r="H45">
+        <v>198</v>
+      </c>
+      <c r="I45">
+        <v>0.434</v>
+      </c>
+      <c r="J45">
+        <v>4</v>
+      </c>
+      <c r="K45">
+        <v>36</v>
+      </c>
+      <c r="L45">
+        <v>15657</v>
+      </c>
+      <c r="M45" s="1">
+        <v>4.3702499999999997E-5</v>
+      </c>
+      <c r="N45">
+        <v>3.2558399999999999E-3</v>
+      </c>
+      <c r="O45">
+        <v>4.3594937185181504</v>
+      </c>
+    </row>
+    <row r="46" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>124</v>
+      </c>
+      <c r="B46" t="s">
+        <v>108</v>
+      </c>
+      <c r="C46" t="s">
+        <v>109</v>
+      </c>
+      <c r="D46">
+        <v>15251</v>
+      </c>
+      <c r="E46" t="s">
+        <v>144</v>
+      </c>
+      <c r="F46" t="s">
+        <v>144</v>
+      </c>
+      <c r="G46">
+        <v>13</v>
+      </c>
+      <c r="H46">
+        <v>24</v>
+      </c>
+      <c r="I46">
+        <v>0.54200000000000004</v>
+      </c>
+      <c r="J46">
+        <v>2</v>
+      </c>
+      <c r="K46">
+        <v>36</v>
+      </c>
+      <c r="L46">
+        <v>15657</v>
+      </c>
+      <c r="M46">
+        <v>3.9460100000000001E-4</v>
+      </c>
+      <c r="N46">
+        <v>1.9598530999999999E-2</v>
+      </c>
+      <c r="O46">
+        <v>3.4038418184910002</v>
+      </c>
+    </row>
+    <row r="47" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>124</v>
+      </c>
+      <c r="B47" t="s">
+        <v>108</v>
+      </c>
+      <c r="C47" t="s">
+        <v>118</v>
+      </c>
+      <c r="D47">
+        <v>15542</v>
+      </c>
+      <c r="E47" t="s">
+        <v>130</v>
+      </c>
+      <c r="F47" t="s">
+        <v>130</v>
+      </c>
+      <c r="G47">
+        <v>85</v>
+      </c>
+      <c r="H47">
+        <v>181</v>
+      </c>
+      <c r="I47">
+        <v>0.47</v>
+      </c>
+      <c r="J47">
+        <v>2</v>
+      </c>
+      <c r="K47">
+        <v>36</v>
+      </c>
+      <c r="L47">
+        <v>15657</v>
+      </c>
+      <c r="M47">
+        <v>1.6282135999999999E-2</v>
+      </c>
+      <c r="N47">
+        <v>9.1966741000000005E-2</v>
+      </c>
+      <c r="O47">
+        <v>1.78828862204124</v>
+      </c>
+    </row>
+    <row r="48" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>124</v>
+      </c>
+      <c r="B48" t="s">
+        <v>108</v>
+      </c>
+      <c r="C48" t="s">
+        <v>118</v>
+      </c>
+      <c r="D48">
+        <v>15580</v>
+      </c>
+      <c r="E48" t="s">
+        <v>127</v>
+      </c>
+      <c r="F48" t="s">
+        <v>127</v>
+      </c>
+      <c r="G48">
+        <v>107</v>
+      </c>
+      <c r="H48">
+        <v>225</v>
+      </c>
+      <c r="I48">
+        <v>0.47599999999999998</v>
+      </c>
+      <c r="J48">
+        <v>2</v>
+      </c>
+      <c r="K48">
+        <v>36</v>
+      </c>
+      <c r="L48">
+        <v>15657</v>
+      </c>
+      <c r="M48">
+        <v>2.5063234E-2</v>
+      </c>
+      <c r="N48">
+        <v>0.109835936</v>
+      </c>
+      <c r="O48">
+        <v>1.6009628911337199</v>
+      </c>
+    </row>
+    <row r="49" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>124</v>
+      </c>
+      <c r="B49" t="s">
+        <v>108</v>
+      </c>
+      <c r="C49" t="s">
+        <v>109</v>
+      </c>
+      <c r="D49">
+        <v>15276</v>
+      </c>
+      <c r="E49" t="s">
+        <v>125</v>
+      </c>
+      <c r="F49" t="s">
+        <v>125</v>
+      </c>
+      <c r="G49">
+        <v>120</v>
+      </c>
+      <c r="H49">
+        <v>304</v>
+      </c>
+      <c r="I49">
+        <v>0.39500000000000002</v>
+      </c>
+      <c r="J49">
+        <v>2</v>
+      </c>
+      <c r="K49">
+        <v>36</v>
+      </c>
+      <c r="L49">
+        <v>15657</v>
+      </c>
+      <c r="M49">
+        <v>3.0975682000000001E-2</v>
+      </c>
+      <c r="N49">
+        <v>0.120458308</v>
+      </c>
+      <c r="O49">
+        <v>1.5089791228671201</v>
+      </c>
+    </row>
+    <row r="50" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>124</v>
+      </c>
+      <c r="B50" t="s">
+        <v>108</v>
+      </c>
+      <c r="C50" t="s">
+        <v>117</v>
+      </c>
+      <c r="D50">
+        <v>15703</v>
+      </c>
+      <c r="E50" t="s">
+        <v>139</v>
+      </c>
+      <c r="F50" t="s">
+        <v>139</v>
+      </c>
+      <c r="G50">
+        <v>15</v>
+      </c>
+      <c r="H50">
+        <v>36</v>
+      </c>
+      <c r="I50">
+        <v>0.41699999999999998</v>
+      </c>
+      <c r="J50">
+        <v>1</v>
+      </c>
+      <c r="K50">
+        <v>36</v>
+      </c>
+      <c r="L50">
+        <v>15657</v>
+      </c>
+      <c r="M50">
+        <v>3.3954691000000002E-2</v>
+      </c>
+      <c r="N50">
+        <v>0.120458308</v>
+      </c>
+      <c r="O50">
+        <v>1.46910021741651</v>
+      </c>
+    </row>
+    <row r="51" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>124</v>
+      </c>
+      <c r="B51" t="s">
+        <v>108</v>
+      </c>
+      <c r="C51" t="s">
+        <v>109</v>
+      </c>
+      <c r="D51">
+        <v>15272</v>
+      </c>
+      <c r="E51" t="s">
+        <v>112</v>
+      </c>
+      <c r="F51" t="s">
+        <v>112</v>
+      </c>
+      <c r="G51">
+        <v>153</v>
+      </c>
+      <c r="H51">
+        <v>430</v>
+      </c>
+      <c r="I51">
+        <v>0.35599999999999998</v>
+      </c>
+      <c r="J51">
+        <v>2</v>
+      </c>
+      <c r="K51">
+        <v>36</v>
+      </c>
+      <c r="L51">
+        <v>15657</v>
+      </c>
+      <c r="M51">
+        <v>4.8133770999999999E-2</v>
+      </c>
+      <c r="N51">
+        <v>0.14725382400000001</v>
+      </c>
+      <c r="O51">
+        <v>1.3175501125520901</v>
+      </c>
+    </row>
+    <row r="52" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>124</v>
+      </c>
+      <c r="B52" t="s">
+        <v>108</v>
+      </c>
+      <c r="C52" t="s">
+        <v>109</v>
+      </c>
+      <c r="D52">
+        <v>15269</v>
+      </c>
+      <c r="E52" t="s">
+        <v>126</v>
+      </c>
+      <c r="F52" t="s">
+        <v>126</v>
+      </c>
+      <c r="G52">
+        <v>174</v>
+      </c>
+      <c r="H52">
+        <v>448</v>
+      </c>
+      <c r="I52">
+        <v>0.38800000000000001</v>
+      </c>
+      <c r="J52">
+        <v>2</v>
+      </c>
+      <c r="K52">
+        <v>36</v>
+      </c>
+      <c r="L52">
+        <v>15657</v>
+      </c>
+      <c r="M52">
+        <v>6.0477632000000003E-2</v>
+      </c>
+      <c r="N52">
+        <v>0.16091369899999999</v>
+      </c>
+      <c r="O52">
+        <v>1.21840522196232</v>
+      </c>
+    </row>
+    <row r="53" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>124</v>
+      </c>
+      <c r="B53" t="s">
+        <v>108</v>
+      </c>
+      <c r="C53" t="s">
+        <v>118</v>
+      </c>
+      <c r="D53">
+        <v>15534</v>
+      </c>
+      <c r="E53" t="s">
+        <v>132</v>
+      </c>
+      <c r="F53" t="s">
+        <v>132</v>
+      </c>
+      <c r="G53">
+        <v>65</v>
+      </c>
+      <c r="H53">
+        <v>141</v>
+      </c>
+      <c r="I53">
+        <v>0.46100000000000002</v>
+      </c>
+      <c r="J53">
+        <v>1</v>
+      </c>
+      <c r="K53">
+        <v>36</v>
+      </c>
+      <c r="L53">
+        <v>15657</v>
+      </c>
+      <c r="M53">
+        <v>0.139234359</v>
+      </c>
+      <c r="N53">
+        <v>0.19941589100000001</v>
+      </c>
+      <c r="O53">
+        <v>0.85625358022256004</v>
+      </c>
+    </row>
+    <row r="54" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
+        <v>124</v>
+      </c>
+      <c r="B54" t="s">
+        <v>108</v>
+      </c>
+      <c r="C54" t="s">
+        <v>109</v>
+      </c>
+      <c r="D54">
+        <v>15153</v>
+      </c>
+      <c r="E54" t="s">
+        <v>135</v>
+      </c>
+      <c r="F54" t="s">
+        <v>135</v>
+      </c>
+      <c r="G54">
+        <v>73</v>
+      </c>
+      <c r="H54">
+        <v>190</v>
+      </c>
+      <c r="I54">
+        <v>0.38400000000000001</v>
+      </c>
+      <c r="J54">
+        <v>1</v>
+      </c>
+      <c r="K54">
+        <v>36</v>
+      </c>
+      <c r="L54">
+        <v>15657</v>
+      </c>
+      <c r="M54">
+        <v>0.15500919199999999</v>
+      </c>
+      <c r="N54">
+        <v>0.20083799699999999</v>
+      </c>
+      <c r="O54">
+        <v>0.80964254752963105</v>
+      </c>
+    </row>
+    <row r="55" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="M55" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C2019F1-6F55-3A40-AF23-59D2C3D3A931}">
   <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -8548,7 +11211,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4125590-F393-A741-AE94-80FB457C9407}">
   <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>

</xml_diff>

<commit_message>
alter curated pathways for c-mwans dot plot
</commit_message>
<xml_diff>
--- a/figures/landscape/curated_pathways.xlsx
+++ b/figures/landscape/curated_pathways.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ch57584/Documents/GitHub/MotrpacPreSuspensionAcute/figures/landscape/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dankatz\Documents\GitHub\MoTrPAC\motrpac-human-presuspension-acute\figures\landscape\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A276099D-D53A-8D43-A496-69538922C979}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCEBF78E-4B4A-4377-B44F-75D23984BAA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7420" yWindow="2160" windowWidth="28040" windowHeight="17180" activeTab="2" xr2:uid="{6CBD5D50-8479-BF41-8318-551E779FC86C}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" activeTab="3" xr2:uid="{6CBD5D50-8479-BF41-8318-551E779FC86C}"/>
   </bookViews>
   <sheets>
     <sheet name="2B" sheetId="1" r:id="rId1"/>
@@ -31,9 +31,10 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -303,9 +304,6 @@
     <t>GOBP_NEUROGENESIS</t>
   </si>
   <si>
-    <t>GOMF_ACTIVE_TRANSMEMBRANE_TRANSPORTER_ACTIVITY</t>
-  </si>
-  <si>
     <t>REFMET_PC</t>
   </si>
   <si>
@@ -351,9 +349,6 @@
     <t>Phosphatidylcholines</t>
   </si>
   <si>
-    <t>Transmembrane Transporters</t>
-  </si>
-  <si>
     <t>Oxidative Phosphorylation</t>
   </si>
   <si>
@@ -475,13 +470,19 @@
   </si>
   <si>
     <t>PTMSIGDB_KINASE-iKiP_MAP2K2</t>
+  </si>
+  <si>
+    <t>GOBP_LYMPHOCYTE_ACTIVATION</t>
+  </si>
+  <si>
+    <t>Lymphocyte Activation</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -848,9 +849,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1CD90C2-1CF4-7D47-8F70-E4845362BEE7}">
   <dimension ref="A1:N17"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14">
       <c r="A1" t="s">
         <v>17</v>
       </c>
@@ -894,7 +895,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:14">
       <c r="A2" t="s">
         <v>30</v>
       </c>
@@ -938,7 +939,7 @@
         <v>17.118207340000001</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:14">
       <c r="A3" t="s">
         <v>30</v>
       </c>
@@ -982,7 +983,7 @@
         <v>16.64636552</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:14">
       <c r="A4" t="s">
         <v>32</v>
       </c>
@@ -1026,7 +1027,7 @@
         <v>16.1530889</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:14">
       <c r="A5" t="s">
         <v>30</v>
       </c>
@@ -1070,7 +1071,7 @@
         <v>15.53245115</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:14">
       <c r="A6" t="s">
         <v>30</v>
       </c>
@@ -1114,7 +1115,7 @@
         <v>14.322972099999999</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:14">
       <c r="A7" t="s">
         <v>30</v>
       </c>
@@ -1158,7 +1159,7 @@
         <v>13.625652909999999</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:14">
       <c r="A8" t="s">
         <v>34</v>
       </c>
@@ -1202,7 +1203,7 @@
         <v>13.512020850000001</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:14">
       <c r="A9" t="s">
         <v>32</v>
       </c>
@@ -1246,7 +1247,7 @@
         <v>12.6904264</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:14">
       <c r="A10" t="s">
         <v>32</v>
       </c>
@@ -1290,7 +1291,7 @@
         <v>12.4666674</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:14">
       <c r="A11" t="s">
         <v>32</v>
       </c>
@@ -1334,7 +1335,7 @@
         <v>11.56752533</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:14">
       <c r="A12" t="s">
         <v>32</v>
       </c>
@@ -1378,7 +1379,7 @@
         <v>10.93094338</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:14">
       <c r="A13" t="s">
         <v>34</v>
       </c>
@@ -1422,7 +1423,7 @@
         <v>10.859424649999999</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:14">
       <c r="A14" t="s">
         <v>30</v>
       </c>
@@ -1466,7 +1467,7 @@
         <v>10.567422369999999</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:14">
       <c r="A15" t="s">
         <v>30</v>
       </c>
@@ -1510,7 +1511,7 @@
         <v>9.8820300920000008</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:14">
       <c r="A16" t="s">
         <v>30</v>
       </c>
@@ -1554,7 +1555,7 @@
         <v>9.0204260470000008</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:14">
       <c r="A17" t="s">
         <v>30</v>
       </c>
@@ -1606,9 +1607,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DBB60F1-11A2-9F42-A04F-2A740A3F7734}">
   <dimension ref="A1:O147"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:15">
       <c r="A1" t="s">
         <v>39</v>
       </c>
@@ -1655,7 +1656,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:15">
       <c r="A2" t="s">
         <v>40</v>
       </c>
@@ -1702,7 +1703,7 @@
         <v>22.228594654156201</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:15">
       <c r="A3" t="s">
         <v>40</v>
       </c>
@@ -1749,7 +1750,7 @@
         <v>16.152479840731999</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:15">
       <c r="A4" t="s">
         <v>40</v>
       </c>
@@ -1796,7 +1797,7 @@
         <v>15.9517211790881</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:15">
       <c r="A5" t="s">
         <v>40</v>
       </c>
@@ -1843,7 +1844,7 @@
         <v>14.8833933185345</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:15">
       <c r="A6" t="s">
         <v>40</v>
       </c>
@@ -1890,7 +1891,7 @@
         <v>14.696699626985</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:15">
       <c r="A7" t="s">
         <v>40</v>
       </c>
@@ -1937,7 +1938,7 @@
         <v>14.263393996823799</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:15">
       <c r="A8" t="s">
         <v>40</v>
       </c>
@@ -1984,7 +1985,7 @@
         <v>13.2037202567479</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:15">
       <c r="A9" t="s">
         <v>40</v>
       </c>
@@ -2031,7 +2032,7 @@
         <v>11.3857484449418</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:15">
       <c r="A10" t="s">
         <v>40</v>
       </c>
@@ -2078,7 +2079,7 @@
         <v>11.3657312661131</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:15">
       <c r="A11" t="s">
         <v>40</v>
       </c>
@@ -2125,7 +2126,7 @@
         <v>10.5875827216032</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:15">
       <c r="A12" t="s">
         <v>40</v>
       </c>
@@ -2172,7 +2173,7 @@
         <v>10.2602250061185</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:15">
       <c r="A13" t="s">
         <v>40</v>
       </c>
@@ -2219,7 +2220,7 @@
         <v>10.185530920524901</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:15">
       <c r="A14" t="s">
         <v>40</v>
       </c>
@@ -2266,7 +2267,7 @@
         <v>9.9318230028991596</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:15">
       <c r="A15" t="s">
         <v>40</v>
       </c>
@@ -2313,7 +2314,7 @@
         <v>9.5576948497478504</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:15">
       <c r="A16" t="s">
         <v>40</v>
       </c>
@@ -2360,7 +2361,7 @@
         <v>8.1683124339608604</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:15">
       <c r="A17" t="s">
         <v>40</v>
       </c>
@@ -2407,7 +2408,7 @@
         <v>8.1298793295998202</v>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:15">
       <c r="A18" t="s">
         <v>40</v>
       </c>
@@ -2454,7 +2455,7 @@
         <v>7.5018958291490998</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:15">
       <c r="A19" t="s">
         <v>40</v>
       </c>
@@ -2501,7 +2502,7 @@
         <v>7.2894174888628296</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:15">
       <c r="A20" t="s">
         <v>40</v>
       </c>
@@ -2548,7 +2549,7 @@
         <v>7.1706110760256001</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:15">
       <c r="A21" t="s">
         <v>40</v>
       </c>
@@ -2595,7 +2596,7 @@
         <v>6.7823277600903804</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:15">
       <c r="A22" t="s">
         <v>40</v>
       </c>
@@ -2642,7 +2643,7 @@
         <v>6.50109373875007</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:15">
       <c r="A23" t="s">
         <v>40</v>
       </c>
@@ -2689,7 +2690,7 @@
         <v>6.4324014260372504</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:15">
       <c r="A24" t="s">
         <v>40</v>
       </c>
@@ -2736,7 +2737,7 @@
         <v>5.94814116964052</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:15">
       <c r="A25" t="s">
         <v>40</v>
       </c>
@@ -2783,7 +2784,7 @@
         <v>5.8425513164437204</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:15">
       <c r="A26" t="s">
         <v>40</v>
       </c>
@@ -2830,7 +2831,7 @@
         <v>5.3677748871384496</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:15">
       <c r="A27" t="s">
         <v>40</v>
       </c>
@@ -2877,7 +2878,7 @@
         <v>5.1557255111947802</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:15">
       <c r="A28" t="s">
         <v>40</v>
       </c>
@@ -2924,7 +2925,7 @@
         <v>4.3781493353569303</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:15">
       <c r="A29" t="s">
         <v>40</v>
       </c>
@@ -2971,7 +2972,7 @@
         <v>3.79298084628399</v>
       </c>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:15">
       <c r="A30" t="s">
         <v>40</v>
       </c>
@@ -3018,7 +3019,7 @@
         <v>3.64060962778324</v>
       </c>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:15">
       <c r="A31" t="s">
         <v>40</v>
       </c>
@@ -3065,7 +3066,7 @@
         <v>3.4908530098817101</v>
       </c>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:15">
       <c r="A32" t="s">
         <v>40</v>
       </c>
@@ -3112,7 +3113,7 @@
         <v>2.1331017299028598</v>
       </c>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:15">
       <c r="A33" t="s">
         <v>40</v>
       </c>
@@ -3159,7 +3160,7 @@
         <v>1.9449251151715501</v>
       </c>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:15">
       <c r="A34" t="s">
         <v>40</v>
       </c>
@@ -3206,7 +3207,7 @@
         <v>1.6667351810717099</v>
       </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:15">
       <c r="A35" t="s">
         <v>40</v>
       </c>
@@ -3253,7 +3254,7 @@
         <v>1.03781860214192</v>
       </c>
     </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:15">
       <c r="A36" t="s">
         <v>75</v>
       </c>
@@ -3300,7 +3301,7 @@
         <v>21.500986722927401</v>
       </c>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:15">
       <c r="A37" t="s">
         <v>75</v>
       </c>
@@ -3347,7 +3348,7 @@
         <v>19.590510594889299</v>
       </c>
     </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:15">
       <c r="A38" t="s">
         <v>75</v>
       </c>
@@ -3394,7 +3395,7 @@
         <v>14.8762706272289</v>
       </c>
     </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:15">
       <c r="A39" t="s">
         <v>75</v>
       </c>
@@ -3441,7 +3442,7 @@
         <v>13.6699551292329</v>
       </c>
     </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:15">
       <c r="A40" t="s">
         <v>75</v>
       </c>
@@ -3488,7 +3489,7 @@
         <v>12.415851285338199</v>
       </c>
     </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:15">
       <c r="A41" t="s">
         <v>75</v>
       </c>
@@ -3535,7 +3536,7 @@
         <v>12.2833792891896</v>
       </c>
     </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:15">
       <c r="A42" t="s">
         <v>75</v>
       </c>
@@ -3582,7 +3583,7 @@
         <v>12.2833792891896</v>
       </c>
     </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:15">
       <c r="A43" t="s">
         <v>75</v>
       </c>
@@ -3629,7 +3630,7 @@
         <v>9.5201832638192201</v>
       </c>
     </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:15">
       <c r="A44" t="s">
         <v>75</v>
       </c>
@@ -3676,7 +3677,7 @@
         <v>9.1601609082192699</v>
       </c>
     </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:15">
       <c r="A45" t="s">
         <v>75</v>
       </c>
@@ -3723,7 +3724,7 @@
         <v>8.9198408135570304</v>
       </c>
     </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:15">
       <c r="A46" t="s">
         <v>75</v>
       </c>
@@ -3770,7 +3771,7 @@
         <v>7.8750504233104301</v>
       </c>
     </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:15">
       <c r="A47" t="s">
         <v>75</v>
       </c>
@@ -3817,7 +3818,7 @@
         <v>7.6983583023314397</v>
       </c>
     </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:15">
       <c r="A48" t="s">
         <v>75</v>
       </c>
@@ -3864,7 +3865,7 @@
         <v>7.3052606987404802</v>
       </c>
     </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:15">
       <c r="A49" t="s">
         <v>75</v>
       </c>
@@ -3911,7 +3912,7 @@
         <v>5.38344324644269</v>
       </c>
     </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:15">
       <c r="A50" t="s">
         <v>75</v>
       </c>
@@ -3958,7 +3959,7 @@
         <v>5.2824729997909001</v>
       </c>
     </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:15">
       <c r="A51" t="s">
         <v>75</v>
       </c>
@@ -4005,7 +4006,7 @@
         <v>4.6062283092758802</v>
       </c>
     </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:15">
       <c r="A52" t="s">
         <v>75</v>
       </c>
@@ -4052,7 +4053,7 @@
         <v>3.90287748981283</v>
       </c>
     </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:15">
       <c r="A53" t="s">
         <v>75</v>
       </c>
@@ -4099,7 +4100,7 @@
         <v>3.4698792545297499</v>
       </c>
     </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:15">
       <c r="A54" t="s">
         <v>75</v>
       </c>
@@ -4146,7 +4147,7 @@
         <v>3.13296266529699</v>
       </c>
     </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:15">
       <c r="A55" t="s">
         <v>75</v>
       </c>
@@ -4193,7 +4194,7 @@
         <v>2.4424889286473102</v>
       </c>
     </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:15">
       <c r="A56" t="s">
         <v>75</v>
       </c>
@@ -4240,7 +4241,7 @@
         <v>2.35597162299901</v>
       </c>
     </row>
-    <row r="57" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:15">
       <c r="A57" t="s">
         <v>75</v>
       </c>
@@ -4287,7 +4288,7 @@
         <v>2.2799378152965</v>
       </c>
     </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:15">
       <c r="A58" t="s">
         <v>75</v>
       </c>
@@ -4334,7 +4335,7 @@
         <v>2.2484381959206901</v>
       </c>
     </row>
-    <row r="59" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:15">
       <c r="A59" t="s">
         <v>75</v>
       </c>
@@ -4381,7 +4382,7 @@
         <v>1.6593687503485399</v>
       </c>
     </row>
-    <row r="60" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:15">
       <c r="A60" t="s">
         <v>75</v>
       </c>
@@ -4428,7 +4429,7 @@
         <v>1.3372205018279899</v>
       </c>
     </row>
-    <row r="61" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:15">
       <c r="A61" t="s">
         <v>75</v>
       </c>
@@ -4475,7 +4476,7 @@
         <v>1.2523873045107301</v>
       </c>
     </row>
-    <row r="62" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:15">
       <c r="A62" t="s">
         <v>75</v>
       </c>
@@ -4522,7 +4523,7 @@
         <v>0.89270764574526396</v>
       </c>
     </row>
-    <row r="63" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:15">
       <c r="A63" t="s">
         <v>75</v>
       </c>
@@ -4569,7 +4570,7 @@
         <v>0.80975257449156302</v>
       </c>
     </row>
-    <row r="64" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:15">
       <c r="A64" t="s">
         <v>75</v>
       </c>
@@ -4616,7 +4617,7 @@
         <v>0.74142892147200301</v>
       </c>
     </row>
-    <row r="65" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:15">
       <c r="A65" t="s">
         <v>75</v>
       </c>
@@ -4663,7 +4664,7 @@
         <v>0.67916752908500699</v>
       </c>
     </row>
-    <row r="66" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:15">
       <c r="A66" t="s">
         <v>75</v>
       </c>
@@ -4710,7 +4711,7 @@
         <v>0.67914318044839395</v>
       </c>
     </row>
-    <row r="67" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:15">
       <c r="A67" t="s">
         <v>75</v>
       </c>
@@ -4757,7 +4758,7 @@
         <v>0.67914318044839395</v>
       </c>
     </row>
-    <row r="68" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:15">
       <c r="A68" t="s">
         <v>75</v>
       </c>
@@ -4804,7 +4805,7 @@
         <v>0.66244781584614298</v>
       </c>
     </row>
-    <row r="69" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:15">
       <c r="A69" t="s">
         <v>75</v>
       </c>
@@ -4851,7 +4852,7 @@
         <v>0.26774750461369201</v>
       </c>
     </row>
-    <row r="70" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:15">
       <c r="A70" t="s">
         <v>76</v>
       </c>
@@ -4898,7 +4899,7 @@
         <v>43.653732495830297</v>
       </c>
     </row>
-    <row r="71" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:15">
       <c r="A71" t="s">
         <v>76</v>
       </c>
@@ -4945,7 +4946,7 @@
         <v>38.422417702297999</v>
       </c>
     </row>
-    <row r="72" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:15">
       <c r="A72" t="s">
         <v>76</v>
       </c>
@@ -4992,7 +4993,7 @@
         <v>31.5295247308322</v>
       </c>
     </row>
-    <row r="73" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:15">
       <c r="A73" t="s">
         <v>76</v>
       </c>
@@ -5039,7 +5040,7 @@
         <v>27.8533619824039</v>
       </c>
     </row>
-    <row r="74" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:15">
       <c r="A74" t="s">
         <v>76</v>
       </c>
@@ -5086,7 +5087,7 @@
         <v>22.32618656372</v>
       </c>
     </row>
-    <row r="75" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:15">
       <c r="A75" t="s">
         <v>76</v>
       </c>
@@ -5133,7 +5134,7 @@
         <v>21.9981476973919</v>
       </c>
     </row>
-    <row r="76" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:15">
       <c r="A76" t="s">
         <v>76</v>
       </c>
@@ -5180,7 +5181,7 @@
         <v>20.317730581275299</v>
       </c>
     </row>
-    <row r="77" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:15">
       <c r="A77" t="s">
         <v>76</v>
       </c>
@@ -5227,7 +5228,7 @@
         <v>20.317730581275299</v>
       </c>
     </row>
-    <row r="78" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:15">
       <c r="A78" t="s">
         <v>76</v>
       </c>
@@ -5274,7 +5275,7 @@
         <v>14.1628941910725</v>
       </c>
     </row>
-    <row r="79" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:15">
       <c r="A79" t="s">
         <v>76</v>
       </c>
@@ -5321,7 +5322,7 @@
         <v>12.8626040441249</v>
       </c>
     </row>
-    <row r="80" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:15">
       <c r="A80" t="s">
         <v>76</v>
       </c>
@@ -5368,7 +5369,7 @@
         <v>12.7316616538736</v>
       </c>
     </row>
-    <row r="81" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:15">
       <c r="A81" t="s">
         <v>76</v>
       </c>
@@ -5415,7 +5416,7 @@
         <v>11.6327682410849</v>
       </c>
     </row>
-    <row r="82" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:15">
       <c r="A82" t="s">
         <v>76</v>
       </c>
@@ -5462,7 +5463,7 @@
         <v>11.6327682410849</v>
       </c>
     </row>
-    <row r="83" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:15">
       <c r="A83" t="s">
         <v>76</v>
       </c>
@@ -5509,7 +5510,7 @@
         <v>11.484739629486</v>
       </c>
     </row>
-    <row r="84" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:15">
       <c r="A84" t="s">
         <v>76</v>
       </c>
@@ -5556,7 +5557,7 @@
         <v>11.195639117676199</v>
       </c>
     </row>
-    <row r="85" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:15">
       <c r="A85" t="s">
         <v>76</v>
       </c>
@@ -5603,7 +5604,7 @@
         <v>10.585641975067</v>
       </c>
     </row>
-    <row r="86" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:15">
       <c r="A86" t="s">
         <v>76</v>
       </c>
@@ -5650,7 +5651,7 @@
         <v>9.6946802804861907</v>
       </c>
     </row>
-    <row r="87" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:15">
       <c r="A87" t="s">
         <v>76</v>
       </c>
@@ -5697,7 +5698,7 @@
         <v>9.2659943665583206</v>
       </c>
     </row>
-    <row r="88" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:15">
       <c r="A88" t="s">
         <v>76</v>
       </c>
@@ -5744,7 +5745,7 @@
         <v>9.1525000452263505</v>
       </c>
     </row>
-    <row r="89" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:15">
       <c r="A89" t="s">
         <v>76</v>
       </c>
@@ -5791,7 +5792,7 @@
         <v>9.0870004318609592</v>
       </c>
     </row>
-    <row r="90" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:15">
       <c r="A90" t="s">
         <v>76</v>
       </c>
@@ -5838,7 +5839,7 @@
         <v>8.5994475408877609</v>
       </c>
     </row>
-    <row r="91" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:15">
       <c r="A91" t="s">
         <v>76</v>
       </c>
@@ -5885,7 +5886,7 @@
         <v>7.6515820150374196</v>
       </c>
     </row>
-    <row r="92" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:15">
       <c r="A92" t="s">
         <v>76</v>
       </c>
@@ -5932,7 +5933,7 @@
         <v>7.4855757772895499</v>
       </c>
     </row>
-    <row r="93" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:15">
       <c r="A93" t="s">
         <v>76</v>
       </c>
@@ -5979,7 +5980,7 @@
         <v>7.4855757772895499</v>
       </c>
     </row>
-    <row r="94" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:15">
       <c r="A94" t="s">
         <v>76</v>
       </c>
@@ -6026,7 +6027,7 @@
         <v>6.5694727845676297</v>
       </c>
     </row>
-    <row r="95" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:15">
       <c r="A95" t="s">
         <v>76</v>
       </c>
@@ -6073,7 +6074,7 @@
         <v>6.0386641129574903</v>
       </c>
     </row>
-    <row r="96" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:15">
       <c r="A96" t="s">
         <v>76</v>
       </c>
@@ -6120,7 +6121,7 @@
         <v>5.8876174335073097</v>
       </c>
     </row>
-    <row r="97" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:15">
       <c r="A97" t="s">
         <v>76</v>
       </c>
@@ -6167,7 +6168,7 @@
         <v>4.77845858661978</v>
       </c>
     </row>
-    <row r="98" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:15">
       <c r="A98" t="s">
         <v>76</v>
       </c>
@@ -6214,7 +6215,7 @@
         <v>4.7422273849187997</v>
       </c>
     </row>
-    <row r="99" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:15">
       <c r="A99" t="s">
         <v>76</v>
       </c>
@@ -6261,7 +6262,7 @@
         <v>4.2650888061166699</v>
       </c>
     </row>
-    <row r="100" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:15">
       <c r="A100" t="s">
         <v>76</v>
       </c>
@@ -6308,7 +6309,7 @@
         <v>2.5344253293096899</v>
       </c>
     </row>
-    <row r="101" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:15">
       <c r="A101" t="s">
         <v>76</v>
       </c>
@@ -6355,7 +6356,7 @@
         <v>2.35894155651894</v>
       </c>
     </row>
-    <row r="102" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:15">
       <c r="A102" t="s">
         <v>76</v>
       </c>
@@ -6402,7 +6403,7 @@
         <v>2.3387399547588599</v>
       </c>
     </row>
-    <row r="103" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:15">
       <c r="A103" t="s">
         <v>76</v>
       </c>
@@ -6449,7 +6450,7 @@
         <v>0.61413247749631095</v>
       </c>
     </row>
-    <row r="104" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:15">
       <c r="A104" t="s">
         <v>77</v>
       </c>
@@ -6496,7 +6497,7 @@
         <v>12.521571037997001</v>
       </c>
     </row>
-    <row r="105" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:15">
       <c r="A105" t="s">
         <v>77</v>
       </c>
@@ -6543,7 +6544,7 @@
         <v>8.2881693283573696</v>
       </c>
     </row>
-    <row r="106" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:15">
       <c r="A106" t="s">
         <v>77</v>
       </c>
@@ -6590,7 +6591,7 @@
         <v>7.6802898745585999</v>
       </c>
     </row>
-    <row r="107" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:15">
       <c r="A107" t="s">
         <v>77</v>
       </c>
@@ -6637,7 +6638,7 @@
         <v>7.4615485074346299</v>
       </c>
     </row>
-    <row r="108" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:15">
       <c r="A108" t="s">
         <v>77</v>
       </c>
@@ -6684,7 +6685,7 @@
         <v>6.9303805934294198</v>
       </c>
     </row>
-    <row r="109" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:15">
       <c r="A109" t="s">
         <v>77</v>
       </c>
@@ -6731,7 +6732,7 @@
         <v>6.3032931331997997</v>
       </c>
     </row>
-    <row r="110" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:15">
       <c r="A110" t="s">
         <v>77</v>
       </c>
@@ -6778,7 +6779,7 @@
         <v>6.2892595682124002</v>
       </c>
     </row>
-    <row r="111" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:15">
       <c r="A111" t="s">
         <v>77</v>
       </c>
@@ -6825,7 +6826,7 @@
         <v>6.2505925647231599</v>
       </c>
     </row>
-    <row r="112" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:15">
       <c r="A112" t="s">
         <v>77</v>
       </c>
@@ -6872,7 +6873,7 @@
         <v>5.9574226070019396</v>
       </c>
     </row>
-    <row r="113" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:15">
       <c r="A113" t="s">
         <v>77</v>
       </c>
@@ -6919,7 +6920,7 @@
         <v>5.68902504816577</v>
       </c>
     </row>
-    <row r="114" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:15">
       <c r="A114" t="s">
         <v>77</v>
       </c>
@@ -6966,7 +6967,7 @@
         <v>5.21321437313365</v>
       </c>
     </row>
-    <row r="115" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:15">
       <c r="A115" t="s">
         <v>77</v>
       </c>
@@ -7013,7 +7014,7 @@
         <v>4.6169203675870802</v>
       </c>
     </row>
-    <row r="116" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:15">
       <c r="A116" t="s">
         <v>77</v>
       </c>
@@ -7060,7 +7061,7 @@
         <v>4.4651356502889303</v>
       </c>
     </row>
-    <row r="117" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:15">
       <c r="A117" t="s">
         <v>77</v>
       </c>
@@ -7107,7 +7108,7 @@
         <v>4.4651356502889303</v>
       </c>
     </row>
-    <row r="118" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:15">
       <c r="A118" t="s">
         <v>77</v>
       </c>
@@ -7154,7 +7155,7 @@
         <v>4.0742237356817101</v>
       </c>
     </row>
-    <row r="119" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:15">
       <c r="A119" t="s">
         <v>77</v>
       </c>
@@ -7201,7 +7202,7 @@
         <v>3.8058580418526899</v>
       </c>
     </row>
-    <row r="120" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:15">
       <c r="A120" t="s">
         <v>77</v>
       </c>
@@ -7248,7 +7249,7 @@
         <v>3.4544011318727601</v>
       </c>
     </row>
-    <row r="121" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:15">
       <c r="A121" t="s">
         <v>77</v>
       </c>
@@ -7295,7 +7296,7 @@
         <v>3.0928023189204801</v>
       </c>
     </row>
-    <row r="122" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:15">
       <c r="A122" t="s">
         <v>77</v>
       </c>
@@ -7342,7 +7343,7 @@
         <v>3.01770170607832</v>
       </c>
     </row>
-    <row r="123" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:15">
       <c r="A123" t="s">
         <v>77</v>
       </c>
@@ -7389,7 +7390,7 @@
         <v>2.89100690830533</v>
       </c>
     </row>
-    <row r="124" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:15">
       <c r="A124" t="s">
         <v>77</v>
       </c>
@@ -7436,7 +7437,7 @@
         <v>2.76604208790534</v>
       </c>
     </row>
-    <row r="125" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:15">
       <c r="A125" t="s">
         <v>77</v>
       </c>
@@ -7483,7 +7484,7 @@
         <v>2.6603531401292702</v>
       </c>
     </row>
-    <row r="126" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:15">
       <c r="A126" t="s">
         <v>77</v>
       </c>
@@ -7530,7 +7531,7 @@
         <v>2.3562552934813898</v>
       </c>
     </row>
-    <row r="127" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:15">
       <c r="A127" t="s">
         <v>77</v>
       </c>
@@ -7577,7 +7578,7 @@
         <v>1.95731635907201</v>
       </c>
     </row>
-    <row r="128" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:15">
       <c r="A128" t="s">
         <v>77</v>
       </c>
@@ -7624,7 +7625,7 @@
         <v>1.9314720967188499</v>
       </c>
     </row>
-    <row r="129" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:15">
       <c r="A129" t="s">
         <v>77</v>
       </c>
@@ -7671,7 +7672,7 @@
         <v>1.2462546975831299</v>
       </c>
     </row>
-    <row r="130" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:15">
       <c r="A130" t="s">
         <v>77</v>
       </c>
@@ -7718,7 +7719,7 @@
         <v>1.16572557019247</v>
       </c>
     </row>
-    <row r="131" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:15">
       <c r="A131" t="s">
         <v>77</v>
       </c>
@@ -7765,7 +7766,7 @@
         <v>0.99659407946909095</v>
       </c>
     </row>
-    <row r="132" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:15">
       <c r="A132" t="s">
         <v>77</v>
       </c>
@@ -7812,7 +7813,7 @@
         <v>0.92577291744546797</v>
       </c>
     </row>
-    <row r="133" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:15">
       <c r="A133" t="s">
         <v>77</v>
       </c>
@@ -7859,7 +7860,7 @@
         <v>0.72936234266796196</v>
       </c>
     </row>
-    <row r="134" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:15">
       <c r="A134" t="s">
         <v>77</v>
       </c>
@@ -7906,7 +7907,7 @@
         <v>0.62353715734978199</v>
       </c>
     </row>
-    <row r="135" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:15">
       <c r="A135" t="s">
         <v>77</v>
       </c>
@@ -7953,7 +7954,7 @@
         <v>0.47925122835905398</v>
       </c>
     </row>
-    <row r="136" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:15">
       <c r="A136" t="s">
         <v>77</v>
       </c>
@@ -8000,7 +8001,7 @@
         <v>0.24823351379941999</v>
       </c>
     </row>
-    <row r="137" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:15">
       <c r="A137" t="s">
         <v>78</v>
       </c>
@@ -8047,7 +8048,7 @@
         <v>8.7979340999613793</v>
       </c>
     </row>
-    <row r="138" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:15">
       <c r="A138" t="s">
         <v>78</v>
       </c>
@@ -8094,7 +8095,7 @@
         <v>5.2929842688503301</v>
       </c>
     </row>
-    <row r="139" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:15">
       <c r="A139" t="s">
         <v>78</v>
       </c>
@@ -8141,7 +8142,7 @@
         <v>3.15639500912713</v>
       </c>
     </row>
-    <row r="140" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:15">
       <c r="A140" t="s">
         <v>78</v>
       </c>
@@ -8188,7 +8189,7 @@
         <v>2.8970509950900598</v>
       </c>
     </row>
-    <row r="141" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:15">
       <c r="A141" t="s">
         <v>78</v>
       </c>
@@ -8235,7 +8236,7 @@
         <v>2.6634399835838098</v>
       </c>
     </row>
-    <row r="142" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:15">
       <c r="A142" t="s">
         <v>78</v>
       </c>
@@ -8282,7 +8283,7 @@
         <v>2.6296053904238099</v>
       </c>
     </row>
-    <row r="143" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:15">
       <c r="A143" t="s">
         <v>78</v>
       </c>
@@ -8329,7 +8330,7 @@
         <v>2.37060269192339</v>
       </c>
     </row>
-    <row r="144" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:15">
       <c r="A144" t="s">
         <v>78</v>
       </c>
@@ -8376,7 +8377,7 @@
         <v>2.2315013857540502</v>
       </c>
     </row>
-    <row r="145" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:15">
       <c r="A145" t="s">
         <v>78</v>
       </c>
@@ -8423,7 +8424,7 @@
         <v>1.94126252135656</v>
       </c>
     </row>
-    <row r="146" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:15">
       <c r="A146" t="s">
         <v>78</v>
       </c>
@@ -8470,7 +8471,7 @@
         <v>1.8126459722089401</v>
       </c>
     </row>
-    <row r="147" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:15">
       <c r="A147" t="s">
         <v>78</v>
       </c>
@@ -8525,9 +8526,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6973C21-7707-B645-8E5F-D6AB2ED24E75}">
   <dimension ref="A1:O55"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:15">
       <c r="A1" t="s">
         <v>39</v>
       </c>
@@ -8574,24 +8575,24 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:15">
       <c r="A2" t="s">
         <v>40</v>
       </c>
       <c r="B2" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D2">
         <v>15276</v>
       </c>
       <c r="E2" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="F2" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="G2">
         <v>120</v>
@@ -8621,24 +8622,24 @@
         <v>12.1946786057447</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:15">
       <c r="A3" t="s">
         <v>40</v>
       </c>
       <c r="B3" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C3" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D3">
         <v>15269</v>
       </c>
       <c r="E3" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="F3" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="G3">
         <v>174</v>
@@ -8668,24 +8669,24 @@
         <v>8.9459311117597498</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:15">
       <c r="A4" t="s">
         <v>40</v>
       </c>
       <c r="B4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C4" t="s">
         <v>108</v>
-      </c>
-      <c r="C4" t="s">
-        <v>110</v>
       </c>
       <c r="D4">
         <v>14946</v>
       </c>
       <c r="E4" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F4" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G4">
         <v>54</v>
@@ -8715,24 +8716,24 @@
         <v>7.9618370215643202</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:15">
       <c r="A5" t="s">
         <v>40</v>
       </c>
       <c r="B5" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C5" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D5">
         <v>15272</v>
       </c>
       <c r="E5" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F5" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="G5">
         <v>153</v>
@@ -8762,24 +8763,24 @@
         <v>7.7551392629791298</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:15">
       <c r="A6" t="s">
         <v>40</v>
       </c>
       <c r="B6" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C6" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D6">
         <v>15580</v>
       </c>
       <c r="E6" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="F6" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="G6">
         <v>107</v>
@@ -8809,24 +8810,24 @@
         <v>7.3048126226907799</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:15">
       <c r="A7" t="s">
         <v>40</v>
       </c>
       <c r="B7" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C7" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="D7">
         <v>15425</v>
       </c>
       <c r="E7" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="F7" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="G7">
         <v>85</v>
@@ -8856,24 +8857,24 @@
         <v>6.77757228762714</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:15">
       <c r="A8" t="s">
         <v>40</v>
       </c>
       <c r="B8" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C8" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D8">
         <v>15542</v>
       </c>
       <c r="E8" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="F8" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="G8">
         <v>85</v>
@@ -8903,24 +8904,24 @@
         <v>5.330752872543</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:15">
       <c r="A9" t="s">
         <v>40</v>
       </c>
       <c r="B9" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C9" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D9">
         <v>14792</v>
       </c>
       <c r="E9" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="F9" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="G9">
         <v>9</v>
@@ -8950,24 +8951,24 @@
         <v>4.0482808195802296</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:15">
       <c r="A10" t="s">
         <v>40</v>
       </c>
       <c r="B10" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C10" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D10">
         <v>14793</v>
       </c>
       <c r="E10" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="F10" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="G10">
         <v>18</v>
@@ -8997,24 +8998,24 @@
         <v>3.7392061844842099</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:15">
       <c r="A11" t="s">
         <v>40</v>
       </c>
       <c r="B11" t="s">
+        <v>106</v>
+      </c>
+      <c r="C11" t="s">
         <v>108</v>
-      </c>
-      <c r="C11" t="s">
-        <v>110</v>
       </c>
       <c r="D11">
         <v>15108</v>
       </c>
       <c r="E11" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="F11" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="G11">
         <v>41</v>
@@ -9044,24 +9045,24 @@
         <v>3.71521971520415</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:15">
       <c r="A12" t="s">
         <v>40</v>
       </c>
       <c r="B12" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C12" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D12">
         <v>15534</v>
       </c>
       <c r="E12" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="F12" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="G12">
         <v>65</v>
@@ -9091,24 +9092,24 @@
         <v>3.5327145907547401</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:15">
       <c r="A13" t="s">
         <v>40</v>
       </c>
       <c r="B13" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C13" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D13">
         <v>15644</v>
       </c>
       <c r="E13" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="F13" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="G13">
         <v>53</v>
@@ -9138,24 +9139,24 @@
         <v>3.13523328255163</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:15">
       <c r="A14" t="s">
         <v>40</v>
       </c>
       <c r="B14" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C14" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D14">
         <v>14776</v>
       </c>
       <c r="E14" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F14" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="G14">
         <v>39</v>
@@ -9185,24 +9186,24 @@
         <v>3.0646464270482898</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:15">
       <c r="A15" t="s">
         <v>40</v>
       </c>
       <c r="B15" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C15" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D15">
         <v>14780</v>
       </c>
       <c r="E15" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="F15" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="G15">
         <v>9</v>
@@ -9232,24 +9233,24 @@
         <v>2.9359038239192299</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:15">
       <c r="A16" t="s">
         <v>40</v>
       </c>
       <c r="B16" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C16" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D16">
         <v>15509</v>
       </c>
       <c r="E16" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="F16" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="G16">
         <v>78</v>
@@ -9279,24 +9280,24 @@
         <v>2.7058416367878801</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:15">
       <c r="A17" t="s">
         <v>40</v>
       </c>
       <c r="B17" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C17" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D17">
         <v>15153</v>
       </c>
       <c r="E17" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="F17" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="G17">
         <v>73</v>
@@ -9326,24 +9327,24 @@
         <v>2.56415881800437</v>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:15">
       <c r="A18" t="s">
         <v>40</v>
       </c>
       <c r="B18" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C18" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D18">
         <v>15708</v>
       </c>
       <c r="E18" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="F18" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="G18">
         <v>28</v>
@@ -9373,24 +9374,24 @@
         <v>2.5219286803068099</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:15">
       <c r="A19" t="s">
         <v>40</v>
       </c>
       <c r="B19" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C19" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="D19">
         <v>15458</v>
       </c>
       <c r="E19" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="F19" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="G19">
         <v>10</v>
@@ -9420,24 +9421,24 @@
         <v>2.5163743384808002</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:15">
       <c r="A20" t="s">
         <v>40</v>
       </c>
       <c r="B20" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C20" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D20">
         <v>15146</v>
       </c>
       <c r="E20" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="F20" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="G20">
         <v>93</v>
@@ -9467,24 +9468,24 @@
         <v>2.5047333944531598</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:15">
       <c r="A21" t="s">
         <v>40</v>
       </c>
       <c r="B21" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C21" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D21">
         <v>15678</v>
       </c>
       <c r="E21" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="F21" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="G21">
         <v>37</v>
@@ -9514,24 +9515,24 @@
         <v>2.4555417622903501</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:15">
       <c r="A22" t="s">
         <v>40</v>
       </c>
       <c r="B22" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C22" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D22">
         <v>15703</v>
       </c>
       <c r="E22" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="F22" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="G22">
         <v>15</v>
@@ -9561,24 +9562,24 @@
         <v>2.4501886474445902</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:15">
       <c r="A23" t="s">
         <v>40</v>
       </c>
       <c r="B23" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C23" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D23">
         <v>15487</v>
       </c>
       <c r="E23" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="F23" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="G23">
         <v>59</v>
@@ -9608,24 +9609,24 @@
         <v>2.36884430027541</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:15">
       <c r="A24" t="s">
         <v>40</v>
       </c>
       <c r="B24" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C24" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D24">
         <v>14844</v>
       </c>
       <c r="E24" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="F24" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="G24">
         <v>13</v>
@@ -9655,24 +9656,24 @@
         <v>2.3135820051533802</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:15">
       <c r="A25" t="s">
         <v>40</v>
       </c>
       <c r="B25" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C25" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="D25">
         <v>15449</v>
       </c>
       <c r="E25" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="F25" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="G25">
         <v>11</v>
@@ -9702,24 +9703,24 @@
         <v>2.1798438777056002</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:15">
       <c r="A26" t="s">
         <v>40</v>
       </c>
       <c r="B26" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C26" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D26">
         <v>15719</v>
       </c>
       <c r="E26" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="F26" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="G26">
         <v>11</v>
@@ -9749,24 +9750,24 @@
         <v>2.1798438777056002</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:15">
       <c r="A27" t="s">
         <v>40</v>
       </c>
       <c r="B27" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C27" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="D27">
         <v>15457</v>
       </c>
       <c r="E27" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="F27" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="G27">
         <v>55</v>
@@ -9796,24 +9797,24 @@
         <v>2.11461039341836</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:15">
       <c r="A28" t="s">
         <v>40</v>
       </c>
       <c r="B28" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C28" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D28">
         <v>15560</v>
       </c>
       <c r="E28" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="F28" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="G28">
         <v>86</v>
@@ -9843,24 +9844,24 @@
         <v>0.58057543104044795</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:15">
       <c r="A29" t="s">
         <v>40</v>
       </c>
       <c r="B29" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C29" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D29">
         <v>15251</v>
       </c>
       <c r="E29" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="F29" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="G29">
         <v>13</v>
@@ -9890,24 +9891,24 @@
         <v>6.3456868742280501E-2</v>
       </c>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:15">
       <c r="A30" t="s">
         <v>77</v>
       </c>
       <c r="B30" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C30" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D30">
         <v>15251</v>
       </c>
       <c r="E30" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="F30" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="G30">
         <v>12</v>
@@ -9937,24 +9938,24 @@
         <v>2.25103419700865</v>
       </c>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:15">
       <c r="A31" t="s">
         <v>77</v>
       </c>
       <c r="B31" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C31" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D31">
         <v>15153</v>
       </c>
       <c r="E31" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="F31" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="G31">
         <v>50</v>
@@ -9984,24 +9985,24 @@
         <v>0.67570970483145198</v>
       </c>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:15">
       <c r="A32" t="s">
         <v>77</v>
       </c>
       <c r="B32" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C32" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="D32">
         <v>15425</v>
       </c>
       <c r="E32" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="F32" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="G32">
         <v>64</v>
@@ -10031,24 +10032,24 @@
         <v>0.47917822661875398</v>
       </c>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:15">
       <c r="A33" t="s">
         <v>77</v>
       </c>
       <c r="B33" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C33" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D33">
         <v>15560</v>
       </c>
       <c r="E33" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="F33" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="G33">
         <v>68</v>
@@ -10078,24 +10079,24 @@
         <v>0.43563172242602899</v>
       </c>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:15">
       <c r="A34" t="s">
         <v>77</v>
       </c>
       <c r="B34" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C34" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="D34">
         <v>15457</v>
       </c>
       <c r="E34" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="F34" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="G34">
         <v>49</v>
@@ -10125,24 +10126,24 @@
         <v>0.33359658721283297</v>
       </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:15">
       <c r="A35" t="s">
         <v>77</v>
       </c>
       <c r="B35" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C35" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D35">
         <v>15534</v>
       </c>
       <c r="E35" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="F35" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="G35">
         <v>50</v>
@@ -10172,24 +10173,24 @@
         <v>0.323842485076622</v>
       </c>
     </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:15">
       <c r="A36" t="s">
         <v>77</v>
       </c>
       <c r="B36" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C36" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D36">
         <v>15487</v>
       </c>
       <c r="E36" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="F36" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="G36">
         <v>51</v>
@@ -10219,24 +10220,24 @@
         <v>0.31441505836627498</v>
       </c>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:15">
       <c r="A37" t="s">
         <v>77</v>
       </c>
       <c r="B37" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C37" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D37">
         <v>15708</v>
       </c>
       <c r="E37" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="F37" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="G37">
         <v>22</v>
@@ -10266,24 +10267,24 @@
         <v>0.29364740719114801</v>
       </c>
     </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:15">
       <c r="A38" t="s">
         <v>77</v>
       </c>
       <c r="B38" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C38" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D38">
         <v>15276</v>
       </c>
       <c r="E38" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="F38" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="G38">
         <v>90</v>
@@ -10313,24 +10314,24 @@
         <v>0.26105922354146499</v>
       </c>
     </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:15">
       <c r="A39" t="s">
         <v>77</v>
       </c>
       <c r="B39" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C39" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D39">
         <v>15509</v>
       </c>
       <c r="E39" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="F39" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="G39">
         <v>59</v>
@@ -10360,24 +10361,24 @@
         <v>0.249235610402569</v>
       </c>
     </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:15">
       <c r="A40" t="s">
         <v>77</v>
       </c>
       <c r="B40" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C40" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D40">
         <v>15269</v>
       </c>
       <c r="E40" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="F40" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="G40">
         <v>127</v>
@@ -10407,24 +10408,24 @@
         <v>0.23859916770530101</v>
       </c>
     </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:15">
       <c r="A41" t="s">
         <v>77</v>
       </c>
       <c r="B41" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C41" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D41">
         <v>15146</v>
       </c>
       <c r="E41" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="F41" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="G41">
         <v>66</v>
@@ -10454,24 +10455,24 @@
         <v>0.20431168293520199</v>
       </c>
     </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:15">
       <c r="A42" t="s">
         <v>77</v>
       </c>
       <c r="B42" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C42" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D42">
         <v>15542</v>
       </c>
       <c r="E42" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="F42" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="G42">
         <v>69</v>
@@ -10501,24 +10502,24 @@
         <v>4.91122598276253E-2</v>
       </c>
     </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:15">
       <c r="A43" t="s">
         <v>77</v>
       </c>
       <c r="B43" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C43" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D43">
         <v>15580</v>
       </c>
       <c r="E43" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="F43" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="G43">
         <v>83</v>
@@ -10548,24 +10549,24 @@
         <v>3.0468432998844001E-2</v>
       </c>
     </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:15">
       <c r="A44" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B44" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C44" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D44">
         <v>15487</v>
       </c>
       <c r="E44" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="F44" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="G44">
         <v>59</v>
@@ -10595,24 +10596,24 @@
         <v>5.0092532421175804</v>
       </c>
     </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:15">
       <c r="A45" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B45" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C45" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D45">
         <v>15560</v>
       </c>
       <c r="E45" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="F45" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="G45">
         <v>86</v>
@@ -10642,24 +10643,24 @@
         <v>4.3594937185181504</v>
       </c>
     </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:15">
       <c r="A46" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B46" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C46" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D46">
         <v>15251</v>
       </c>
       <c r="E46" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="F46" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="G46">
         <v>13</v>
@@ -10689,24 +10690,24 @@
         <v>3.4038418184910002</v>
       </c>
     </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:15">
       <c r="A47" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B47" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C47" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D47">
         <v>15542</v>
       </c>
       <c r="E47" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="F47" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="G47">
         <v>85</v>
@@ -10736,24 +10737,24 @@
         <v>1.78828862204124</v>
       </c>
     </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:15">
       <c r="A48" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B48" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C48" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D48">
         <v>15580</v>
       </c>
       <c r="E48" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="F48" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="G48">
         <v>107</v>
@@ -10783,24 +10784,24 @@
         <v>1.6009628911337199</v>
       </c>
     </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:15">
       <c r="A49" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B49" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C49" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D49">
         <v>15276</v>
       </c>
       <c r="E49" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="F49" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="G49">
         <v>120</v>
@@ -10830,24 +10831,24 @@
         <v>1.5089791228671201</v>
       </c>
     </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:15">
       <c r="A50" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B50" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C50" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D50">
         <v>15703</v>
       </c>
       <c r="E50" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="F50" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="G50">
         <v>15</v>
@@ -10877,24 +10878,24 @@
         <v>1.46910021741651</v>
       </c>
     </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:15">
       <c r="A51" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B51" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C51" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D51">
         <v>15272</v>
       </c>
       <c r="E51" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F51" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="G51">
         <v>153</v>
@@ -10924,24 +10925,24 @@
         <v>1.3175501125520901</v>
       </c>
     </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:15">
       <c r="A52" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B52" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C52" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D52">
         <v>15269</v>
       </c>
       <c r="E52" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="F52" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="G52">
         <v>174</v>
@@ -10971,24 +10972,24 @@
         <v>1.21840522196232</v>
       </c>
     </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:15">
       <c r="A53" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B53" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C53" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D53">
         <v>15534</v>
       </c>
       <c r="E53" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="F53" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="G53">
         <v>65</v>
@@ -11018,24 +11019,24 @@
         <v>0.85625358022256004</v>
       </c>
     </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:15">
       <c r="A54" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B54" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C54" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D54">
         <v>15153</v>
       </c>
       <c r="E54" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="F54" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="G54">
         <v>73</v>
@@ -11065,7 +11066,7 @@
         <v>0.80964254752963105</v>
       </c>
     </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:15">
       <c r="M55" s="1"/>
     </row>
   </sheetData>
@@ -11076,97 +11077,97 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C2019F1-6F55-3A40-AF23-59D2C3D3A931}">
   <dimension ref="A1:B16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2">
       <c r="A1" t="s">
         <v>16</v>
       </c>
       <c r="B1" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
       <c r="A2" t="s">
         <v>79</v>
       </c>
       <c r="B2" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
       <c r="A3" t="s">
         <v>80</v>
       </c>
       <c r="B3" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
       <c r="A4" t="s">
         <v>81</v>
       </c>
       <c r="B4" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
       <c r="A5" t="s">
         <v>82</v>
       </c>
       <c r="B5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
       <c r="A6" t="s">
         <v>50</v>
       </c>
       <c r="B6" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
       <c r="A7" t="s">
         <v>83</v>
       </c>
       <c r="B7" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
       <c r="A8" t="s">
         <v>84</v>
       </c>
       <c r="B8" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
       <c r="A9" t="s">
         <v>85</v>
       </c>
       <c r="B9" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
       <c r="A10" t="s">
         <v>86</v>
       </c>
       <c r="B10" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
       <c r="A11" t="s">
         <v>87</v>
       </c>
       <c r="B11" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
       <c r="A12" t="s">
         <v>88</v>
       </c>
@@ -11174,36 +11175,36 @@
         <v>102</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:2">
       <c r="A13" t="s">
         <v>89</v>
       </c>
       <c r="B13" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
       <c r="A14" t="s">
-        <v>90</v>
+        <v>143</v>
       </c>
       <c r="B14" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
       <c r="A15" t="s">
         <v>9</v>
       </c>
       <c r="B15" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2">
       <c r="A16" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B16" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
   </sheetData>
@@ -11214,89 +11215,89 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4125590-F393-A741-AE94-80FB457C9407}">
   <dimension ref="A1:A17"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:1">
       <c r="A1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:1">
       <c r="A2">
         <v>12955</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:1">
       <c r="A3">
         <v>1798</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:1">
       <c r="A4">
         <v>10098</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:1">
       <c r="A5">
         <v>7678</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:1">
       <c r="A6">
         <v>573</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:1">
       <c r="A7">
         <v>12940</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:1">
       <c r="A8">
         <v>135</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:1">
       <c r="A9">
         <v>4838</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:1">
       <c r="A10">
         <v>14364</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:1">
       <c r="A11">
         <v>2065</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:1">
       <c r="A12">
         <v>7757</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:1">
       <c r="A13">
         <v>3898</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:1">
       <c r="A14">
         <v>12753</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:1">
       <c r="A15">
         <v>983</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:1">
       <c r="A16">
         <v>6315</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:1">
       <c r="A17">
         <v>14323</v>
       </c>

</xml_diff>